<commit_message>
Complete Milestone 0 novelty audit and preregistration
</commit_message>
<xml_diff>
--- a/Literature/literature_matrix.xlsx
+++ b/Literature/literature_matrix.xlsx
@@ -2,11 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literature Matrix" sheetId="1" r:id="Rb8b0c228b76742e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batch 02 Additions" sheetId="2" r:id="R0ad680082dfc454b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Novelty Map" sheetId="3" r:id="R2c36c590f2a846b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestone Status" sheetId="4" r:id="Rfefc58083ef3410a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="5" r:id="Rc8422378956644ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literature Matrix" sheetId="1" r:id="R0fdc016453924e31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status" sheetId="2" r:id="R4004bb3017274469"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +14,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="5">
+  <x:fonts count="4">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -40,14 +37,8 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FF274E13"/>
-      <x:name val="Carlito"/>
-    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -67,11 +58,6 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF2F75B5"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFD9EAD3"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -138,7 +124,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="79">
+  <x:cellXfs count="73">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -308,29 +294,11 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="7">
+  <x:dxfs count="3">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -362,216 +330,12 @@
         </x:patternFill>
       </x:fill>
     </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF9C0006"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFF4CCCC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF7F6000"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFFF2CC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF274E13"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFD9EAD3"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF9C0006"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFF4CCCC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
 
-<file path=xl/drawings/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:r>
-              <a:rPr/>
-              <a:t>Cumulative Sources by Literature Family</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:overlay val="0"/>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:v>Sources</c:v>
-          </c:tx>
-          <c:cat>
-            <c:strRef>
-              <c:f>'Milestone Status'!$A$13:$A$20</c:f>
-              <c:strCache>
-                <c:ptCount val="0"/>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'Milestone Status'!$B$13:$B$20</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="0"/>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-          <c:showLeaderLines val="0"/>
-        </c:dLbls>
-        <c:axId val="48650112"/>
-        <c:axId val="48672768"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="48650112"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="CCCCCC"/>
-              </a:solidFill>
-              <a:prstDash val="dash"/>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="48672768"/>
-        <c:crosses val="autoZero"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="48672768"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="CCCCCC"/>
-              </a:solidFill>
-              <a:prstDash val="dash"/>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:crossAx val="48650112"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-  </c:chart>
-  <c:spPr>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-      <a:solidFill>
-        <a:srgbClr val="D9D9D9"/>
-      </a:solidFill>
-      <a:prstDash val="solid"/>
-    </a:ln>
-  </c:spPr>
-</c:chartSpace>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="1" name="Chart"/>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
-        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R51875b516aca4de9"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LiteratureMatrixBatch02" displayName="LiteratureMatrixBatch02" ref="A4:Q65" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LiteratureMatrixV03" displayName="LiteratureMatrixV03" ref="A4:Q66" headerRowCount="1">
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Theme"/>
@@ -590,43 +354,6 @@
     <x:tableColumn id="15" name="Source URL"/>
     <x:tableColumn id="16" name="Verification"/>
     <x:tableColumn id="17" name="Last Checked"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Batch02Additions" displayName="Batch02Additions" ref="A4:Q35" headerRowCount="1">
-  <x:tableColumns count="17">
-    <x:tableColumn id="1" name="ID"/>
-    <x:tableColumn id="2" name="Theme"/>
-    <x:tableColumn id="3" name="Citation Key"/>
-    <x:tableColumn id="4" name="Authors"/>
-    <x:tableColumn id="5" name="Year"/>
-    <x:tableColumn id="6" name="Title"/>
-    <x:tableColumn id="7" name="Outlet / Status"/>
-    <x:tableColumn id="8" name="Document / Data"/>
-    <x:tableColumn id="9" name="Method"/>
-    <x:tableColumn id="10" name="Outcome / Task"/>
-    <x:tableColumn id="11" name="Key Finding"/>
-    <x:tableColumn id="12" name="Overlap with Disclosure Drift"/>
-    <x:tableColumn id="13" name="Novelty Threat"/>
-    <x:tableColumn id="14" name="Planned Use"/>
-    <x:tableColumn id="15" name="Source URL"/>
-    <x:tableColumn id="16" name="Verification"/>
-    <x:tableColumn id="17" name="Last Checked"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="NoveltyBoundaryTable" displayName="NoveltyBoundaryTable" ref="A3:D10" headerRowCount="1">
-  <x:tableColumns count="4">
-    <x:tableColumn id="1" name="Potential claim"/>
-    <x:tableColumn id="2" name="Closest competing source(s)"/>
-    <x:tableColumn id="3" name="Status after Batch 02"/>
-    <x:tableColumn id="4" name="Required project distinction"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </x:table>
@@ -788,21 +515,21 @@
     <x:col min="5" max="5" width="9" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="44" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="27" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="36" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="29" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="42" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="44" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="35" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="38" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="30" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="44" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="46" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="40" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="39" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="24" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="41" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="38" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="27" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>Disclosure Drift — Cumulative Literature Matrix through Batch 02</x:v>
+        <x:v>Disclosure Drift — Literature Matrix v0.3</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -821,9 +548,9 @@
       <x:c r="P1" s="4"/>
       <x:c r="Q1" s="4"/>
     </x:row>
-    <x:row r="2" ht="36" customHeight="1">
+    <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="11" t="str">
-        <x:v>61 verified high-priority, adjacent, and foundational sources. The CSV is the repository’s authoritative machine-readable matrix; this workbook is the review copy.</x:v>
+        <x:v>62-source cumulative matrix. Adds Choi (2026) after the direct-competitor literature refresh.</x:v>
       </x:c>
       <x:c r="B2" s="11"/>
       <x:c r="C2" s="11"/>
@@ -895,7 +622,7 @@
         <x:v>Last Checked</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="82" customHeight="1">
+    <x:row r="5" ht="80" customHeight="1">
       <x:c r="A5" s="58" t="str">
         <x:v>DRIFT-01</x:v>
       </x:c>
@@ -948,7 +675,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="82" customHeight="1">
+    <x:row r="6" ht="80" customHeight="1">
       <x:c r="A6" s="58" t="str">
         <x:v>GENAI-01</x:v>
       </x:c>
@@ -1001,7 +728,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="82" customHeight="1">
+    <x:row r="7" ht="80" customHeight="1">
       <x:c r="A7" s="58" t="str">
         <x:v>DRIFT-02</x:v>
       </x:c>
@@ -1054,7 +781,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="82" customHeight="1">
+    <x:row r="8" ht="80" customHeight="1">
       <x:c r="A8" s="58" t="str">
         <x:v>GENAI-02</x:v>
       </x:c>
@@ -1107,7 +834,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="82" customHeight="1">
+    <x:row r="9" ht="80" customHeight="1">
       <x:c r="A9" s="58" t="str">
         <x:v>GENAI-03</x:v>
       </x:c>
@@ -1160,7 +887,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="82" customHeight="1">
+    <x:row r="10" ht="80" customHeight="1">
       <x:c r="A10" s="58" t="str">
         <x:v>GENAI-04</x:v>
       </x:c>
@@ -1213,7 +940,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="82" customHeight="1">
+    <x:row r="11" ht="80" customHeight="1">
       <x:c r="A11" s="58" t="str">
         <x:v>REWRITE-01</x:v>
       </x:c>
@@ -1266,7 +993,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="82" customHeight="1">
+    <x:row r="12" ht="80" customHeight="1">
       <x:c r="A12" s="58" t="str">
         <x:v>GENAI-05</x:v>
       </x:c>
@@ -1319,7 +1046,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="82" customHeight="1">
+    <x:row r="13" ht="80" customHeight="1">
       <x:c r="A13" s="58" t="str">
         <x:v>DRIFT-03</x:v>
       </x:c>
@@ -1372,7 +1099,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="82" customHeight="1">
+    <x:row r="14" ht="80" customHeight="1">
       <x:c r="A14" s="58" t="str">
         <x:v>BASE-01</x:v>
       </x:c>
@@ -1425,7 +1152,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="82" customHeight="1">
+    <x:row r="15" ht="80" customHeight="1">
       <x:c r="A15" s="58" t="str">
         <x:v>BASE-02</x:v>
       </x:c>
@@ -1478,7 +1205,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="82" customHeight="1">
+    <x:row r="16" ht="80" customHeight="1">
       <x:c r="A16" s="58" t="str">
         <x:v>BASE-03</x:v>
       </x:c>
@@ -1531,7 +1258,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="82" customHeight="1">
+    <x:row r="17" ht="80" customHeight="1">
       <x:c r="A17" s="58" t="str">
         <x:v>BASE-04</x:v>
       </x:c>
@@ -1584,7 +1311,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="82" customHeight="1">
+    <x:row r="18" ht="80" customHeight="1">
       <x:c r="A18" s="58" t="str">
         <x:v>BASE-05</x:v>
       </x:c>
@@ -1637,7 +1364,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="82" customHeight="1">
+    <x:row r="19" ht="80" customHeight="1">
       <x:c r="A19" s="58" t="str">
         <x:v>BASE-06</x:v>
       </x:c>
@@ -1690,7 +1417,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="82" customHeight="1">
+    <x:row r="20" ht="80" customHeight="1">
       <x:c r="A20" s="58" t="str">
         <x:v>BASE-07</x:v>
       </x:c>
@@ -1743,7 +1470,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="82" customHeight="1">
+    <x:row r="21" ht="80" customHeight="1">
       <x:c r="A21" s="58" t="str">
         <x:v>BASE-08</x:v>
       </x:c>
@@ -1796,7 +1523,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="82" customHeight="1">
+    <x:row r="22" ht="80" customHeight="1">
       <x:c r="A22" s="58" t="str">
         <x:v>BASE-09</x:v>
       </x:c>
@@ -1849,7 +1576,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="82" customHeight="1">
+    <x:row r="23" ht="80" customHeight="1">
       <x:c r="A23" s="58" t="str">
         <x:v>BASE-10</x:v>
       </x:c>
@@ -1902,7 +1629,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="82" customHeight="1">
+    <x:row r="24" ht="80" customHeight="1">
       <x:c r="A24" s="58" t="str">
         <x:v>PRED-01</x:v>
       </x:c>
@@ -1955,7 +1682,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="82" customHeight="1">
+    <x:row r="25" ht="80" customHeight="1">
       <x:c r="A25" s="58" t="str">
         <x:v>DATA-01</x:v>
       </x:c>
@@ -2008,7 +1735,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="82" customHeight="1">
+    <x:row r="26" ht="80" customHeight="1">
       <x:c r="A26" s="58" t="str">
         <x:v>NLP-01</x:v>
       </x:c>
@@ -2061,7 +1788,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="82" customHeight="1">
+    <x:row r="27" ht="80" customHeight="1">
       <x:c r="A27" s="58" t="str">
         <x:v>GROUND-01</x:v>
       </x:c>
@@ -2114,7 +1841,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="82" customHeight="1">
+    <x:row r="28" ht="80" customHeight="1">
       <x:c r="A28" s="58" t="str">
         <x:v>GROUND-02</x:v>
       </x:c>
@@ -2167,7 +1894,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="82" customHeight="1">
+    <x:row r="29" ht="80" customHeight="1">
       <x:c r="A29" s="58" t="str">
         <x:v>CAL-01</x:v>
       </x:c>
@@ -2220,7 +1947,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="82" customHeight="1">
+    <x:row r="30" ht="80" customHeight="1">
       <x:c r="A30" s="58" t="str">
         <x:v>SHIFT-01</x:v>
       </x:c>
@@ -2273,7 +2000,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="82" customHeight="1">
+    <x:row r="31" ht="80" customHeight="1">
       <x:c r="A31" s="58" t="str">
         <x:v>CAL-02</x:v>
       </x:c>
@@ -2326,7 +2053,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="82" customHeight="1">
+    <x:row r="32" ht="80" customHeight="1">
       <x:c r="A32" s="58" t="str">
         <x:v>DETECT-01</x:v>
       </x:c>
@@ -2379,7 +2106,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="82" customHeight="1">
+    <x:row r="33" ht="80" customHeight="1">
       <x:c r="A33" s="58" t="str">
         <x:v>DETECT-02</x:v>
       </x:c>
@@ -2432,7 +2159,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="82" customHeight="1">
+    <x:row r="34" ht="80" customHeight="1">
       <x:c r="A34" s="58" t="str">
         <x:v>DETECT-03</x:v>
       </x:c>
@@ -2485,7 +2212,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="82" customHeight="1">
+    <x:row r="35" ht="80" customHeight="1">
       <x:c r="A35" s="58" t="str">
         <x:v>BASE-11</x:v>
       </x:c>
@@ -2498,7 +2225,7 @@
       <x:c r="D35" s="59" t="str">
         <x:v>Brown, Stephen V.; Tucker, Jennifer Wu</x:v>
       </x:c>
-      <x:c r="E35" s="59" t="n">
+      <x:c r="E35" s="59" t="str">
         <x:v>2011</x:v>
       </x:c>
       <x:c r="F35" s="59" t="str">
@@ -2538,7 +2265,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="82" customHeight="1">
+    <x:row r="36" ht="80" customHeight="1">
       <x:c r="A36" s="58" t="str">
         <x:v>BASE-12</x:v>
       </x:c>
@@ -2551,7 +2278,7 @@
       <x:c r="D36" s="59" t="str">
         <x:v>Feldman, Ronen; Govindaraj, Suresh; Livnat, Joshua; Segal, Benjamin</x:v>
       </x:c>
-      <x:c r="E36" s="59" t="n">
+      <x:c r="E36" s="59" t="str">
         <x:v>2010</x:v>
       </x:c>
       <x:c r="F36" s="59" t="str">
@@ -2591,7 +2318,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="82" customHeight="1">
+    <x:row r="37" ht="80" customHeight="1">
       <x:c r="A37" s="58" t="str">
         <x:v>BASE-13</x:v>
       </x:c>
@@ -2604,7 +2331,7 @@
       <x:c r="D37" s="59" t="str">
         <x:v>Kravet, Todd D.; Muslu, Volkan</x:v>
       </x:c>
-      <x:c r="E37" s="59" t="n">
+      <x:c r="E37" s="59" t="str">
         <x:v>2013</x:v>
       </x:c>
       <x:c r="F37" s="59" t="str">
@@ -2644,7 +2371,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="82" customHeight="1">
+    <x:row r="38" ht="80" customHeight="1">
       <x:c r="A38" s="58" t="str">
         <x:v>BASE-14</x:v>
       </x:c>
@@ -2657,7 +2384,7 @@
       <x:c r="D38" s="59" t="str">
         <x:v>Bao, Yang; Datta, Anindya</x:v>
       </x:c>
-      <x:c r="E38" s="59" t="n">
+      <x:c r="E38" s="59" t="str">
         <x:v>2014</x:v>
       </x:c>
       <x:c r="F38" s="59" t="str">
@@ -2697,7 +2424,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="82" customHeight="1">
+    <x:row r="39" ht="80" customHeight="1">
       <x:c r="A39" s="58" t="str">
         <x:v>BASE-15</x:v>
       </x:c>
@@ -2710,7 +2437,7 @@
       <x:c r="D39" s="59" t="str">
         <x:v>Hope, Ole-Kristian; Hu, Danqi; Lu, Hai</x:v>
       </x:c>
-      <x:c r="E39" s="59" t="n">
+      <x:c r="E39" s="59" t="str">
         <x:v>2016</x:v>
       </x:c>
       <x:c r="F39" s="59" t="str">
@@ -2750,7 +2477,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="82" customHeight="1">
+    <x:row r="40" ht="80" customHeight="1">
       <x:c r="A40" s="58" t="str">
         <x:v>BASE-16</x:v>
       </x:c>
@@ -2763,7 +2490,7 @@
       <x:c r="D40" s="59" t="str">
         <x:v>Dyer, Travis; Lang, Mark; Stice-Lawrence, Lorien</x:v>
       </x:c>
-      <x:c r="E40" s="59" t="n">
+      <x:c r="E40" s="59" t="str">
         <x:v>2017</x:v>
       </x:c>
       <x:c r="F40" s="59" t="str">
@@ -2803,7 +2530,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="82" customHeight="1">
+    <x:row r="41" ht="80" customHeight="1">
       <x:c r="A41" s="58" t="str">
         <x:v>PRED-02</x:v>
       </x:c>
@@ -2816,7 +2543,7 @@
       <x:c r="D41" s="59" t="str">
         <x:v>Cohen, Lauren; Malloy, Christopher J.; Nguyen, Quoc H.</x:v>
       </x:c>
-      <x:c r="E41" s="59" t="n">
+      <x:c r="E41" s="59" t="str">
         <x:v>2020</x:v>
       </x:c>
       <x:c r="F41" s="59" t="str">
@@ -2856,7 +2583,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" ht="82" customHeight="1">
+    <x:row r="42" ht="80" customHeight="1">
       <x:c r="A42" s="58" t="str">
         <x:v>PRED-03</x:v>
       </x:c>
@@ -2869,7 +2596,7 @@
       <x:c r="D42" s="59" t="str">
         <x:v>Kogan, Shimon; Levin, Dimitry; Routledge, Bryan R.; Sagi, Jacob S.; Smith, Noah A.</x:v>
       </x:c>
-      <x:c r="E42" s="59" t="n">
+      <x:c r="E42" s="59" t="str">
         <x:v>2009</x:v>
       </x:c>
       <x:c r="F42" s="59" t="str">
@@ -2909,7 +2636,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="82" customHeight="1">
+    <x:row r="43" ht="80" customHeight="1">
       <x:c r="A43" s="58" t="str">
         <x:v>PRED-04</x:v>
       </x:c>
@@ -2922,7 +2649,7 @@
       <x:c r="D43" s="59" t="str">
         <x:v>Sedinkina, Marina; Breitkopf, Nikolas; Schütze, Hinrich</x:v>
       </x:c>
-      <x:c r="E43" s="59" t="n">
+      <x:c r="E43" s="59" t="str">
         <x:v>2019</x:v>
       </x:c>
       <x:c r="F43" s="59" t="str">
@@ -2962,7 +2689,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="44" ht="82" customHeight="1">
+    <x:row r="44" ht="80" customHeight="1">
       <x:c r="A44" s="58" t="str">
         <x:v>PRED-05</x:v>
       </x:c>
@@ -2975,7 +2702,7 @@
       <x:c r="D44" s="59" t="str">
         <x:v>Tsai, Ming-Feng; Wang, Chuan-Ju</x:v>
       </x:c>
-      <x:c r="E44" s="59" t="n">
+      <x:c r="E44" s="59" t="str">
         <x:v>2017</x:v>
       </x:c>
       <x:c r="F44" s="59" t="str">
@@ -3015,7 +2742,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="45" ht="82" customHeight="1">
+    <x:row r="45" ht="80" customHeight="1">
       <x:c r="A45" s="58" t="str">
         <x:v>REVIEW-01</x:v>
       </x:c>
@@ -3028,7 +2755,7 @@
       <x:c r="D45" s="59" t="str">
         <x:v>Bochkay, Khrystyna; Brown, Stephen V.; Leone, Andrew J.; Tucker, Jennifer Wu</x:v>
       </x:c>
-      <x:c r="E45" s="59" t="n">
+      <x:c r="E45" s="59" t="str">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="F45" s="59" t="str">
@@ -3068,7 +2795,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="82" customHeight="1">
+    <x:row r="46" ht="80" customHeight="1">
       <x:c r="A46" s="58" t="str">
         <x:v>PRED-06</x:v>
       </x:c>
@@ -3081,7 +2808,7 @@
       <x:c r="D46" s="59" t="str">
         <x:v>Bogachek, Olga; De Vito, Antonio; Demeré, Paul; Grossetti, Francesco</x:v>
       </x:c>
-      <x:c r="E46" s="59" t="n">
+      <x:c r="E46" s="59" t="str">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="F46" s="59" t="str">
@@ -3121,7 +2848,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="47" ht="82" customHeight="1">
+    <x:row r="47" ht="80" customHeight="1">
       <x:c r="A47" s="58" t="str">
         <x:v>PRED-07</x:v>
       </x:c>
@@ -3134,7 +2861,7 @@
       <x:c r="D47" s="59" t="str">
         <x:v>Kim, Alex G.; Muhn, Maximilian; Nikolaev, Valeri V.; Zhang, Yijing</x:v>
       </x:c>
-      <x:c r="E47" s="59" t="n">
+      <x:c r="E47" s="59" t="str">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="F47" s="59" t="str">
@@ -3174,7 +2901,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="48" ht="82" customHeight="1">
+    <x:row r="48" ht="80" customHeight="1">
       <x:c r="A48" s="58" t="str">
         <x:v>PRED-08</x:v>
       </x:c>
@@ -3187,7 +2914,7 @@
       <x:c r="D48" s="59" t="str">
         <x:v>Gupta, Aparna; Rawte, Vipula; Zaki, Mohammed J.</x:v>
       </x:c>
-      <x:c r="E48" s="59" t="n">
+      <x:c r="E48" s="59" t="str">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="F48" s="59" t="str">
@@ -3227,7 +2954,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="82" customHeight="1">
+    <x:row r="49" ht="80" customHeight="1">
       <x:c r="A49" s="58" t="str">
         <x:v>PRED-09</x:v>
       </x:c>
@@ -3240,7 +2967,7 @@
       <x:c r="D49" s="59" t="str">
         <x:v>Grundy, Bruce D.; Petry, Stefan</x:v>
       </x:c>
-      <x:c r="E49" s="59" t="n">
+      <x:c r="E49" s="59" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F49" s="59" t="str">
@@ -3280,7 +3007,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="50" ht="82" customHeight="1">
+    <x:row r="50" ht="80" customHeight="1">
       <x:c r="A50" s="58" t="str">
         <x:v>PRED-10</x:v>
       </x:c>
@@ -3293,7 +3020,7 @@
       <x:c r="D50" s="59" t="str">
         <x:v>Zhang, Zhen; Zheng, Moxuan; Zhang, Tongchen; Lin, Luyun; Wang, Yiqing; Lin, Lixing</x:v>
       </x:c>
-      <x:c r="E50" s="59" t="n">
+      <x:c r="E50" s="59" t="str">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="F50" s="59" t="str">
@@ -3333,7 +3060,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="51" ht="82" customHeight="1">
+    <x:row r="51" ht="80" customHeight="1">
       <x:c r="A51" s="58" t="str">
         <x:v>PRED-11</x:v>
       </x:c>
@@ -3346,7 +3073,7 @@
       <x:c r="D51" s="59" t="str">
         <x:v>Lin, Tom</x:v>
       </x:c>
-      <x:c r="E51" s="59" t="n">
+      <x:c r="E51" s="59" t="str">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="F51" s="59" t="str">
@@ -3386,7 +3113,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="52" ht="82" customHeight="1">
+    <x:row r="52" ht="80" customHeight="1">
       <x:c r="A52" s="58" t="str">
         <x:v>BASE-17</x:v>
       </x:c>
@@ -3399,7 +3126,7 @@
       <x:c r="D52" s="59" t="str">
         <x:v>Chin, Michael; Liu, Yue; Moffitt, Kevin</x:v>
       </x:c>
-      <x:c r="E52" s="59" t="n">
+      <x:c r="E52" s="59" t="str">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="F52" s="59" t="str">
@@ -3439,7 +3166,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="53" ht="82" customHeight="1">
+    <x:row r="53" ht="80" customHeight="1">
       <x:c r="A53" s="58" t="str">
         <x:v>DISC-01</x:v>
       </x:c>
@@ -3452,7 +3179,7 @@
       <x:c r="D53" s="59" t="str">
         <x:v>Blann, James Justin; Moon, James R.; Wang, Yuxiao</x:v>
       </x:c>
-      <x:c r="E53" s="59" t="n">
+      <x:c r="E53" s="59" t="str">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="F53" s="59" t="str">
@@ -3492,7 +3219,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" ht="82" customHeight="1">
+    <x:row r="54" ht="80" customHeight="1">
       <x:c r="A54" s="58" t="str">
         <x:v>GENAI-06</x:v>
       </x:c>
@@ -3505,7 +3232,7 @@
       <x:c r="D54" s="59" t="str">
         <x:v>Jia, Ning; Li, Ningzhong; Xu, Da; Zhang, Yuwen</x:v>
       </x:c>
-      <x:c r="E54" s="59" t="n">
+      <x:c r="E54" s="59" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F54" s="59" t="str">
@@ -3545,7 +3272,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="55" ht="82" customHeight="1">
+    <x:row r="55" ht="80" customHeight="1">
       <x:c r="A55" s="58" t="str">
         <x:v>GENAI-07</x:v>
       </x:c>
@@ -3558,7 +3285,7 @@
       <x:c r="D55" s="59" t="str">
         <x:v>Jia, Ning; Li, Ningzhong; Ma, Guang; Xu, Da</x:v>
       </x:c>
-      <x:c r="E55" s="59" t="n">
+      <x:c r="E55" s="59" t="str">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="F55" s="59" t="str">
@@ -3598,7 +3325,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="56" ht="82" customHeight="1">
+    <x:row r="56" ht="80" customHeight="1">
       <x:c r="A56" s="58" t="str">
         <x:v>GENAI-08</x:v>
       </x:c>
@@ -3611,7 +3338,7 @@
       <x:c r="D56" s="59" t="str">
         <x:v>Cho, Tony; Huang, Allen H.; Pacelli, Joseph; Rennekamp, Kristina</x:v>
       </x:c>
-      <x:c r="E56" s="59" t="n">
+      <x:c r="E56" s="59" t="str">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="F56" s="59" t="str">
@@ -3651,7 +3378,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" ht="82" customHeight="1">
+    <x:row r="57" ht="80" customHeight="1">
       <x:c r="A57" s="58" t="str">
         <x:v>GENAI-09</x:v>
       </x:c>
@@ -3664,7 +3391,7 @@
       <x:c r="D57" s="59" t="str">
         <x:v>Cao, Sean Shun; Chen, Wilbur Xinyuan; Ma, Guang; Srinivasan, Suraj</x:v>
       </x:c>
-      <x:c r="E57" s="59" t="n">
+      <x:c r="E57" s="59" t="str">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="F57" s="59" t="str">
@@ -3704,7 +3431,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="58" ht="82" customHeight="1">
+    <x:row r="58" ht="80" customHeight="1">
       <x:c r="A58" s="58" t="str">
         <x:v>GENAI-10</x:v>
       </x:c>
@@ -3717,7 +3444,7 @@
       <x:c r="D58" s="59" t="str">
         <x:v>Marin, Lucas G. Uberti-Bona; Rijsbosch, Bram; Spanakis, Gerasimos; Kollnig, Konrad</x:v>
       </x:c>
-      <x:c r="E58" s="59" t="n">
+      <x:c r="E58" s="59" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F58" s="59" t="str">
@@ -3757,7 +3484,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="59" ht="82" customHeight="1">
+    <x:row r="59" ht="80" customHeight="1">
       <x:c r="A59" s="58" t="str">
         <x:v>GROUND-03</x:v>
       </x:c>
@@ -3770,7 +3497,7 @@
       <x:c r="D59" s="59" t="str">
         <x:v>Wang, Ruilong; Balloccu, Simone</x:v>
       </x:c>
-      <x:c r="E59" s="59" t="n">
+      <x:c r="E59" s="59" t="str">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="F59" s="59" t="str">
@@ -3810,7 +3537,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="60" ht="82" customHeight="1">
+    <x:row r="60" ht="80" customHeight="1">
       <x:c r="A60" s="58" t="str">
         <x:v>GROUND-04</x:v>
       </x:c>
@@ -3823,7 +3550,7 @@
       <x:c r="D60" s="59" t="str">
         <x:v>Panda, Silu</x:v>
       </x:c>
-      <x:c r="E60" s="59" t="n">
+      <x:c r="E60" s="59" t="str">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="F60" s="59" t="str">
@@ -3863,7 +3590,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="61" ht="82" customHeight="1">
+    <x:row r="61" ht="80" customHeight="1">
       <x:c r="A61" s="58" t="str">
         <x:v>GROUND-05</x:v>
       </x:c>
@@ -3876,7 +3603,7 @@
       <x:c r="D61" s="59" t="str">
         <x:v>Dolphin, Robert; Dursun, Irem; Blankenship, Jeff; Adams, Griffin; Pike, Christopher</x:v>
       </x:c>
-      <x:c r="E61" s="59" t="n">
+      <x:c r="E61" s="59" t="str">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="F61" s="59" t="str">
@@ -3916,7 +3643,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="62" ht="82" customHeight="1">
+    <x:row r="62" ht="80" customHeight="1">
       <x:c r="A62" s="58" t="str">
         <x:v>DATA-02</x:v>
       </x:c>
@@ -3929,7 +3656,7 @@
       <x:c r="D62" s="59" t="str">
         <x:v>Bettencourt, Jesse; Ding, Yuxuan; Giesecke, Kay</x:v>
       </x:c>
-      <x:c r="E62" s="59" t="n">
+      <x:c r="E62" s="59" t="str">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="F62" s="59" t="str">
@@ -3969,7 +3696,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="63" ht="82" customHeight="1">
+    <x:row r="63" ht="80" customHeight="1">
       <x:c r="A63" s="58" t="str">
         <x:v>GROUND-06</x:v>
       </x:c>
@@ -3982,7 +3709,7 @@
       <x:c r="D63" s="59" t="str">
         <x:v>Long, Yicheng; Hu, Yifan; Zhao, Yilun; Cohan, Arman; Zhao, Yilun</x:v>
       </x:c>
-      <x:c r="E63" s="59" t="n">
+      <x:c r="E63" s="59" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="F63" s="59" t="str">
@@ -4022,7 +3749,7 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="64" ht="82" customHeight="1">
+    <x:row r="64" ht="80" customHeight="1">
       <x:c r="A64" s="58" t="str">
         <x:v>GROUND-07</x:v>
       </x:c>
@@ -4035,7 +3762,7 @@
       <x:c r="D64" s="59" t="str">
         <x:v>Guo, Yuchen; Wu, Shijie; Yiu, Siu-Ming</x:v>
       </x:c>
-      <x:c r="E64" s="59" t="n">
+      <x:c r="E64" s="59" t="str">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="F64" s="59" t="str">
@@ -4075,56 +3802,109 @@
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
-    <x:row r="65" ht="82" customHeight="1">
-      <x:c r="A65" s="61" t="str">
+    <x:row r="65" ht="80" customHeight="1">
+      <x:c r="A65" s="58" t="str">
         <x:v>GROUND-08</x:v>
       </x:c>
-      <x:c r="B65" s="62" t="str">
+      <x:c r="B65" s="59" t="str">
         <x:v>Financial multi-document RAG benchmark</x:v>
       </x:c>
-      <x:c r="C65" s="62" t="str">
+      <x:c r="C65" s="59" t="str">
         <x:v>yang2026finmragbench</x:v>
       </x:c>
-      <x:c r="D65" s="62" t="str">
+      <x:c r="D65" s="59" t="str">
         <x:v>Yang, Yucheng; Zhang, Yiming; Li, Zhenyu; Chen, Qian; Wang, Haoyu; Liu, Zhiyuan</x:v>
       </x:c>
-      <x:c r="E65" s="62" t="n">
+      <x:c r="E65" s="59" t="str">
         <x:v>2026</x:v>
       </x:c>
-      <x:c r="F65" s="62" t="str">
+      <x:c r="F65" s="59" t="str">
         <x:v>FinMRAGBench: Benchmarking Multi-Document Retrieval-Augmented Generation in Finance</x:v>
       </x:c>
-      <x:c r="G65" s="62" t="str">
+      <x:c r="G65" s="59" t="str">
         <x:v>Findings of ACL 2026</x:v>
       </x:c>
-      <x:c r="H65" s="62" t="str">
+      <x:c r="H65" s="59" t="str">
         <x:v>Multiple financial documents and evidence-intensive questions</x:v>
       </x:c>
-      <x:c r="I65" s="62" t="str">
+      <x:c r="I65" s="59" t="str">
         <x:v>Retrieval-augmented generation benchmark</x:v>
       </x:c>
-      <x:c r="J65" s="62" t="str">
+      <x:c r="J65" s="59" t="str">
         <x:v>Multi-document financial reasoning and attribution</x:v>
       </x:c>
-      <x:c r="K65" s="62" t="str">
+      <x:c r="K65" s="59" t="str">
         <x:v>Shows the difficulty of retrieving and synthesizing the correct evidence across financial documents.</x:v>
       </x:c>
-      <x:c r="L65" s="62" t="str">
+      <x:c r="L65" s="59" t="str">
         <x:v>Supports rigorous source retrieval and evidence coverage in the robust model.</x:v>
       </x:c>
-      <x:c r="M65" s="62" t="str">
+      <x:c r="M65" s="59" t="str">
         <x:v>Low</x:v>
       </x:c>
-      <x:c r="N65" s="62" t="str">
+      <x:c r="N65" s="59" t="str">
         <x:v>Multi-source evidence and citation evaluation.</x:v>
       </x:c>
-      <x:c r="O65" s="62" t="str">
+      <x:c r="O65" s="59" t="str">
         <x:v>https://aclanthology.org/2026.findings-acl.187/</x:v>
       </x:c>
-      <x:c r="P65" s="62" t="str">
+      <x:c r="P65" s="59" t="str">
         <x:v>Primary ACL metadata reviewed</x:v>
       </x:c>
-      <x:c r="Q65" s="63" t="str">
+      <x:c r="Q65" s="60" t="str">
+        <x:v>2026-07-25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="80" customHeight="1">
+      <x:c r="A66" s="61" t="str">
+        <x:v>PRED-12</x:v>
+      </x:c>
+      <x:c r="B66" s="62" t="str">
+        <x:v>Aggregation-dependent 10-K sentiment</x:v>
+      </x:c>
+      <x:c r="C66" s="62" t="str">
+        <x:v>choi2026howmuch</x:v>
+      </x:c>
+      <x:c r="D66" s="62" t="str">
+        <x:v>Choi, Sanggyu Sean</x:v>
+      </x:c>
+      <x:c r="E66" s="62" t="str">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="F66" s="62" t="str">
+        <x:v>How Much of a 10-K Matters? Aggregation-Dependent Value of Full-Text versus Risk-Factor Sentiment</x:v>
+      </x:c>
+      <x:c r="G66" s="62" t="str">
+        <x:v>arXiv preprint</x:v>
+      </x:c>
+      <x:c r="H66" s="62" t="str">
+        <x:v>1,383 10-K filings from 94 Nasdaq-100 technology constituents, 2006–2023</x:v>
+      </x:c>
+      <x:c r="I66" s="62" t="str">
+        <x:v>Supervised lexicon learning against return and volatility labels at sector, portfolio, and individual-firm aggregation levels</x:v>
+      </x:c>
+      <x:c r="J66" s="62" t="str">
+        <x:v>Return and realized-volatility sentiment classification and correlation with market outcomes</x:v>
+      </x:c>
+      <x:c r="K66" s="62" t="str">
+        <x:v>Full-filing text performs better at sector and portfolio levels, while Item 1A performs better at the individual-firm level; the result depends on aggregation and available training signal.</x:v>
+      </x:c>
+      <x:c r="L66" s="62" t="str">
+        <x:v>Important late-breaking comparator for full-text versus section-specific modeling and supervised 10-K language measures, but not a GenAI-era temporal reliability, calibration, operating-outcome, or rewrite study.</x:v>
+      </x:c>
+      <x:c r="M66" s="62" t="str">
+        <x:v>Medium-High</x:v>
+      </x:c>
+      <x:c r="N66" s="62" t="str">
+        <x:v>Require section-specific and aggregation-level robustness checks; avoid claiming novelty for comparing full 10-K text with Item 1A.</x:v>
+      </x:c>
+      <x:c r="O66" s="62" t="str">
+        <x:v>https://arxiv.org/abs/2607.14174</x:v>
+      </x:c>
+      <x:c r="P66" s="62" t="str">
+        <x:v>Full primary arXiv paper reviewed</x:v>
+      </x:c>
+      <x:c r="Q66" s="63" t="str">
         <x:v>2026-07-25</x:v>
       </x:c>
     </x:row>
@@ -4133,7 +3913,7 @@
     <x:mergeCell ref="A1:Q1"/>
     <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="M5:M65">
+  <x:conditionalFormatting sqref="M5:M66">
     <x:cfRule type="expression" dxfId="0" priority="1">
       <x:formula>OR(M5="High",LEFT(M5,4)="High")</x:formula>
     </x:cfRule>
@@ -4146,7 +3926,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ff71c2225694755"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7fed057a32c434f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4155,2191 +3935,56 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="31" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="9" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="44" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="27" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="36" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="29" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="42" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="44" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="40" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="39" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="24" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="4" t="str">
-        <x:v>Disclosure Drift — Literature Batch 02 Additions</x:v>
-      </x:c>
-      <x:c r="B1" s="4"/>
-      <x:c r="C1" s="4"/>
-      <x:c r="D1" s="4"/>
-      <x:c r="E1" s="4"/>
-      <x:c r="F1" s="4"/>
-      <x:c r="G1" s="4"/>
-      <x:c r="H1" s="4"/>
-      <x:c r="I1" s="4"/>
-      <x:c r="J1" s="4"/>
-      <x:c r="K1" s="4"/>
-      <x:c r="L1" s="4"/>
-      <x:c r="M1" s="4"/>
-      <x:c r="N1" s="4"/>
-      <x:c r="O1" s="4"/>
-      <x:c r="P1" s="4"/>
-      <x:c r="Q1" s="4"/>
-    </x:row>
-    <x:row r="2" ht="36" customHeight="1">
-      <x:c r="A2" s="11" t="str">
-        <x:v>31 sources added through direct-competitor review, backward/forward citation chaining, and evidence-grounding searches.</x:v>
-      </x:c>
-      <x:c r="B2" s="11"/>
-      <x:c r="C2" s="11"/>
-      <x:c r="D2" s="11"/>
-      <x:c r="E2" s="11"/>
-      <x:c r="F2" s="11"/>
-      <x:c r="G2" s="11"/>
-      <x:c r="H2" s="11"/>
-      <x:c r="I2" s="11"/>
-      <x:c r="J2" s="11"/>
-      <x:c r="K2" s="11"/>
-      <x:c r="L2" s="11"/>
-      <x:c r="M2" s="11"/>
-      <x:c r="N2" s="11"/>
-      <x:c r="O2" s="11"/>
-      <x:c r="P2" s="11"/>
-      <x:c r="Q2" s="11"/>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="55" t="str">
-        <x:v>ID</x:v>
-      </x:c>
-      <x:c r="B4" s="56" t="str">
-        <x:v>Theme</x:v>
-      </x:c>
-      <x:c r="C4" s="56" t="str">
-        <x:v>Citation Key</x:v>
-      </x:c>
-      <x:c r="D4" s="56" t="str">
-        <x:v>Authors</x:v>
-      </x:c>
-      <x:c r="E4" s="56" t="str">
-        <x:v>Year</x:v>
-      </x:c>
-      <x:c r="F4" s="56" t="str">
-        <x:v>Title</x:v>
-      </x:c>
-      <x:c r="G4" s="56" t="str">
-        <x:v>Outlet / Status</x:v>
-      </x:c>
-      <x:c r="H4" s="56" t="str">
-        <x:v>Document / Data</x:v>
-      </x:c>
-      <x:c r="I4" s="56" t="str">
-        <x:v>Method</x:v>
-      </x:c>
-      <x:c r="J4" s="56" t="str">
-        <x:v>Outcome / Task</x:v>
-      </x:c>
-      <x:c r="K4" s="56" t="str">
-        <x:v>Key Finding</x:v>
-      </x:c>
-      <x:c r="L4" s="56" t="str">
-        <x:v>Overlap with Disclosure Drift</x:v>
-      </x:c>
-      <x:c r="M4" s="56" t="str">
-        <x:v>Novelty Threat</x:v>
-      </x:c>
-      <x:c r="N4" s="56" t="str">
-        <x:v>Planned Use</x:v>
-      </x:c>
-      <x:c r="O4" s="56" t="str">
-        <x:v>Source URL</x:v>
-      </x:c>
-      <x:c r="P4" s="56" t="str">
-        <x:v>Verification</x:v>
-      </x:c>
-      <x:c r="Q4" s="57" t="str">
-        <x:v>Last Checked</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="82" customHeight="1">
-      <x:c r="A5" s="58" t="str">
-        <x:v>BASE-11</x:v>
-      </x:c>
-      <x:c r="B5" s="59" t="str">
-        <x:v>Year-over-year MD&amp;A change</x:v>
-      </x:c>
-      <x:c r="C5" s="59" t="str">
-        <x:v>brown2011mdachanges</x:v>
-      </x:c>
-      <x:c r="D5" s="59" t="str">
-        <x:v>Brown, Stephen V.; Tucker, Jennifer Wu</x:v>
-      </x:c>
-      <x:c r="E5" s="59" t="n">
-        <x:v>2011</x:v>
-      </x:c>
-      <x:c r="F5" s="59" t="str">
-        <x:v>Large-Sample Evidence on Firms’ Year-over-Year MD&amp;A Modifications</x:v>
-      </x:c>
-      <x:c r="G5" s="59" t="str">
-        <x:v>Journal of Accounting Research</x:v>
-      </x:c>
-      <x:c r="H5" s="59" t="str">
-        <x:v>Management’s Discussion and Analysis sections</x:v>
-      </x:c>
-      <x:c r="I5" s="59" t="str">
-        <x:v>Year-over-year textual modification scores and capital-market tests</x:v>
-      </x:c>
-      <x:c r="J5" s="59" t="str">
-        <x:v>Economic change, filing reactions, and disclosure usefulness</x:v>
-      </x:c>
-      <x:c r="K5" s="59" t="str">
-        <x:v>MD&amp;A modification captures economically meaningful disclosure change, while the usefulness of modification measures can vary over time.</x:v>
-      </x:c>
-      <x:c r="L5" s="59" t="str">
-        <x:v>Foundational precedent for longitudinal disclosure-change and similarity features.</x:v>
-      </x:c>
-      <x:c r="M5" s="59" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="N5" s="59" t="str">
-        <x:v>Required year-over-year similarity baseline and interpretation guide.</x:v>
-      </x:c>
-      <x:c r="O5" s="59" t="str">
-        <x:v>https://doi.org/10.1111/j.1475-679X.2010.00396.x</x:v>
-      </x:c>
-      <x:c r="P5" s="59" t="str">
-        <x:v>Primary journal page reviewed</x:v>
-      </x:c>
-      <x:c r="Q5" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="82" customHeight="1">
-      <x:c r="A6" s="58" t="str">
-        <x:v>BASE-12</x:v>
-      </x:c>
-      <x:c r="B6" s="59" t="str">
-        <x:v>MD&amp;A tone change</x:v>
-      </x:c>
-      <x:c r="C6" s="59" t="str">
-        <x:v>feldman2010tone</x:v>
-      </x:c>
-      <x:c r="D6" s="59" t="str">
-        <x:v>Feldman, Ronen; Govindaraj, Suresh; Livnat, Joshua; Segal, Benjamin</x:v>
-      </x:c>
-      <x:c r="E6" s="59" t="n">
-        <x:v>2010</x:v>
-      </x:c>
-      <x:c r="F6" s="59" t="str">
-        <x:v>Management’s Tone Change, Post Earnings Announcement Drift and Accruals</x:v>
-      </x:c>
-      <x:c r="G6" s="59" t="str">
-        <x:v>Review of Accounting Studies</x:v>
-      </x:c>
-      <x:c r="H6" s="59" t="str">
-        <x:v>MD&amp;A sections of Forms 10-K and 10-Q</x:v>
-      </x:c>
-      <x:c r="I6" s="59" t="str">
-        <x:v>Tone-change measures combined with financial controls</x:v>
-      </x:c>
-      <x:c r="J6" s="59" t="str">
-        <x:v>Post-announcement returns and incremental disclosure information</x:v>
-      </x:c>
-      <x:c r="K6" s="59" t="str">
-        <x:v>Changes in management tone contain information beyond contemporaneous financial measures.</x:v>
-      </x:c>
-      <x:c r="L6" s="59" t="str">
-        <x:v>Canonical tone-change baseline that could become unstable when drafting style changes.</x:v>
-      </x:c>
-      <x:c r="M6" s="59" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="N6" s="59" t="str">
-        <x:v>Traditional tone-change benchmark.</x:v>
-      </x:c>
-      <x:c r="O6" s="59" t="str">
-        <x:v>https://ssrn.com/abstract=1287083</x:v>
-      </x:c>
-      <x:c r="P6" s="59" t="str">
-        <x:v>Primary SSRN page reviewed</x:v>
-      </x:c>
-      <x:c r="Q6" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="82" customHeight="1">
-      <x:c r="A7" s="58" t="str">
-        <x:v>BASE-13</x:v>
-      </x:c>
-      <x:c r="B7" s="59" t="str">
-        <x:v>Risk disclosure change</x:v>
-      </x:c>
-      <x:c r="C7" s="59" t="str">
-        <x:v>kravet2013risk</x:v>
-      </x:c>
-      <x:c r="D7" s="59" t="str">
-        <x:v>Kravet, Todd D.; Muslu, Volkan</x:v>
-      </x:c>
-      <x:c r="E7" s="59" t="n">
-        <x:v>2013</x:v>
-      </x:c>
-      <x:c r="F7" s="59" t="str">
-        <x:v>Textual Risk Disclosures and Investors’ Risk Perceptions</x:v>
-      </x:c>
-      <x:c r="G7" s="59" t="str">
-        <x:v>Review of Accounting Studies</x:v>
-      </x:c>
-      <x:c r="H7" s="59" t="str">
-        <x:v>10-K textual risk disclosures</x:v>
-      </x:c>
-      <x:c r="I7" s="59" t="str">
-        <x:v>Disclosure-change measures and market/analyst responses</x:v>
-      </x:c>
-      <x:c r="J7" s="59" t="str">
-        <x:v>Trading, volatility, and investor risk perception</x:v>
-      </x:c>
-      <x:c r="K7" s="59" t="str">
-        <x:v>Changes in risk disclosure are associated with changes in investor risk perceptions.</x:v>
-      </x:c>
-      <x:c r="L7" s="59" t="str">
-        <x:v>Foundational Item 1A change measure and risk-language benchmark.</x:v>
-      </x:c>
-      <x:c r="M7" s="59" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="N7" s="59" t="str">
-        <x:v>Risk-section baseline and falsification design.</x:v>
-      </x:c>
-      <x:c r="O7" s="59" t="str">
-        <x:v>https://doi.org/10.1007/s11142-013-9228-9</x:v>
-      </x:c>
-      <x:c r="P7" s="59" t="str">
-        <x:v>Primary bibliographic and journal metadata reviewed</x:v>
-      </x:c>
-      <x:c r="Q7" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="82" customHeight="1">
-      <x:c r="A8" s="58" t="str">
-        <x:v>BASE-14</x:v>
-      </x:c>
-      <x:c r="B8" s="59" t="str">
-        <x:v>Risk-topic discovery</x:v>
-      </x:c>
-      <x:c r="C8" s="59" t="str">
-        <x:v>bao2014risktypes</x:v>
-      </x:c>
-      <x:c r="D8" s="59" t="str">
-        <x:v>Bao, Yang; Datta, Anindya</x:v>
-      </x:c>
-      <x:c r="E8" s="59" t="n">
-        <x:v>2014</x:v>
-      </x:c>
-      <x:c r="F8" s="59" t="str">
-        <x:v>Simultaneously Discovering and Quantifying Risk Types from Textual Risk Disclosures</x:v>
-      </x:c>
-      <x:c r="G8" s="59" t="str">
-        <x:v>Management Science</x:v>
-      </x:c>
-      <x:c r="H8" s="59" t="str">
-        <x:v>Corporate textual risk disclosures</x:v>
-      </x:c>
-      <x:c r="I8" s="59" t="str">
-        <x:v>Topic modeling for discovery and quantification of risk types</x:v>
-      </x:c>
-      <x:c r="J8" s="59" t="str">
-        <x:v>Risk-type measurement and investor perceptions</x:v>
-      </x:c>
-      <x:c r="K8" s="59" t="str">
-        <x:v>Distinct textual risk categories can be discovered and linked differently to perceived risk.</x:v>
-      </x:c>
-      <x:c r="L8" s="59" t="str">
-        <x:v>Precedent for interpretable risk-topic components rather than one aggregate tone score.</x:v>
-      </x:c>
-      <x:c r="M8" s="59" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="N8" s="59" t="str">
-        <x:v>Risk taxonomy and component-level feature audit.</x:v>
-      </x:c>
-      <x:c r="O8" s="59" t="str">
-        <x:v>https://doi.org/10.1287/mnsc.2014.1930</x:v>
-      </x:c>
-      <x:c r="P8" s="59" t="str">
-        <x:v>Primary journal page reviewed</x:v>
-      </x:c>
-      <x:c r="Q8" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="82" customHeight="1">
-      <x:c r="A9" s="58" t="str">
-        <x:v>BASE-15</x:v>
-      </x:c>
-      <x:c r="B9" s="59" t="str">
-        <x:v>Risk specificity</x:v>
-      </x:c>
-      <x:c r="C9" s="59" t="str">
-        <x:v>hope2016specific</x:v>
-      </x:c>
-      <x:c r="D9" s="59" t="str">
-        <x:v>Hope, Ole-Kristian; Hu, Danqi; Lu, Hai</x:v>
-      </x:c>
-      <x:c r="E9" s="59" t="n">
-        <x:v>2016</x:v>
-      </x:c>
-      <x:c r="F9" s="59" t="str">
-        <x:v>The Benefits of Specific Risk-Factor Disclosures</x:v>
-      </x:c>
-      <x:c r="G9" s="59" t="str">
-        <x:v>Review of Accounting Studies</x:v>
-      </x:c>
-      <x:c r="H9" s="59" t="str">
-        <x:v>Item 1A risk-factor disclosures</x:v>
-      </x:c>
-      <x:c r="I9" s="59" t="str">
-        <x:v>Specificity measures and capital-market analyses</x:v>
-      </x:c>
-      <x:c r="J9" s="59" t="str">
-        <x:v>Disclosure informativeness and market outcomes</x:v>
-      </x:c>
-      <x:c r="K9" s="59" t="str">
-        <x:v>More specific risk-factor disclosures are more informative than generic risk language.</x:v>
-      </x:c>
-      <x:c r="L9" s="59" t="str">
-        <x:v>Supports firm-specific term density and claim-specificity components.</x:v>
-      </x:c>
-      <x:c r="M9" s="59" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="N9" s="59" t="str">
-        <x:v>Specificity baseline and evidence-grounding definition.</x:v>
-      </x:c>
-      <x:c r="O9" s="59" t="str">
-        <x:v>https://doi.org/10.1007/s11142-016-9371-1</x:v>
-      </x:c>
-      <x:c r="P9" s="59" t="str">
-        <x:v>Primary journal metadata reviewed</x:v>
-      </x:c>
-      <x:c r="Q9" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="82" customHeight="1">
-      <x:c r="A10" s="58" t="str">
-        <x:v>BASE-16</x:v>
-      </x:c>
-      <x:c r="B10" s="59" t="str">
-        <x:v>Long-run 10-K evolution</x:v>
-      </x:c>
-      <x:c r="C10" s="59" t="str">
-        <x:v>dyer2017evolution</x:v>
-      </x:c>
-      <x:c r="D10" s="59" t="str">
-        <x:v>Dyer, Travis; Lang, Mark; Stice-Lawrence, Lorien</x:v>
-      </x:c>
-      <x:c r="E10" s="59" t="n">
-        <x:v>2017</x:v>
-      </x:c>
-      <x:c r="F10" s="59" t="str">
-        <x:v>The Evolution of 10-K Textual Disclosure: Evidence from Latent Dirichlet Allocation</x:v>
-      </x:c>
-      <x:c r="G10" s="59" t="str">
-        <x:v>Journal of Accounting and Economics</x:v>
-      </x:c>
-      <x:c r="H10" s="59" t="str">
-        <x:v>Large historical corpus of 10-K filings</x:v>
-      </x:c>
-      <x:c r="I10" s="59" t="str">
-        <x:v>Topic modeling and longitudinal disclosure analysis</x:v>
-      </x:c>
-      <x:c r="J10" s="59" t="str">
-        <x:v>Long-run evolution in filing topics and properties</x:v>
-      </x:c>
-      <x:c r="K10" s="59" t="str">
-        <x:v>10-K disclosure content and structure evolve materially over long horizons.</x:v>
-      </x:c>
-      <x:c r="L10" s="59" t="str">
-        <x:v>Critical warning that post-2022 differences must be separated from ordinary long-run evolution.</x:v>
-      </x:c>
-      <x:c r="M10" s="59" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="N10" s="59" t="str">
-        <x:v>Pretrend modeling, placebo cutoffs, and historical context.</x:v>
-      </x:c>
-      <x:c r="O10" s="59" t="str">
-        <x:v>https://doi.org/10.1016/j.jacceco.2017.07.002</x:v>
-      </x:c>
-      <x:c r="P10" s="59" t="str">
-        <x:v>Primary journal metadata reviewed</x:v>
-      </x:c>
-      <x:c r="Q10" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="82" customHeight="1">
-      <x:c r="A11" s="58" t="str">
-        <x:v>PRED-02</x:v>
-      </x:c>
-      <x:c r="B11" s="59" t="str">
-        <x:v>Disclosure change and future returns</x:v>
-      </x:c>
-      <x:c r="C11" s="59" t="str">
-        <x:v>cohen2020lazyprices</x:v>
-      </x:c>
-      <x:c r="D11" s="59" t="str">
-        <x:v>Cohen, Lauren; Malloy, Christopher J.; Nguyen, Quoc H.</x:v>
-      </x:c>
-      <x:c r="E11" s="59" t="n">
-        <x:v>2020</x:v>
-      </x:c>
-      <x:c r="F11" s="59" t="str">
-        <x:v>Lazy Prices</x:v>
-      </x:c>
-      <x:c r="G11" s="59" t="str">
-        <x:v>Journal of Finance</x:v>
-      </x:c>
-      <x:c r="H11" s="59" t="str">
-        <x:v>Corporate filing text and year-over-year disclosure changes</x:v>
-      </x:c>
-      <x:c r="I11" s="59" t="str">
-        <x:v>Textual change measures and asset-pricing tests</x:v>
-      </x:c>
-      <x:c r="J11" s="59" t="str">
-        <x:v>Future stock returns</x:v>
-      </x:c>
-      <x:c r="K11" s="59" t="str">
-        <x:v>Changes in corporate filings contain predictive information that markets may process slowly.</x:v>
-      </x:c>
-      <x:c r="L11" s="59" t="str">
-        <x:v>Major precedent for predictive power in disclosure changes.</x:v>
-      </x:c>
-      <x:c r="M11" s="59" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="N11" s="59" t="str">
-        <x:v>Similarity/change benchmark while distinguishing operating outcomes from returns.</x:v>
-      </x:c>
-      <x:c r="O11" s="59" t="str">
-        <x:v>https://doi.org/10.1111/jofi.12885</x:v>
-      </x:c>
-      <x:c r="P11" s="59" t="str">
-        <x:v>Primary journal metadata reviewed</x:v>
-      </x:c>
-      <x:c r="Q11" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="82" customHeight="1">
-      <x:c r="A12" s="58" t="str">
-        <x:v>PRED-03</x:v>
-      </x:c>
-      <x:c r="B12" s="59" t="str">
-        <x:v>Text-based risk prediction</x:v>
-      </x:c>
-      <x:c r="C12" s="59" t="str">
-        <x:v>kogan2009risk</x:v>
-      </x:c>
-      <x:c r="D12" s="59" t="str">
-        <x:v>Kogan, Shimon; Levin, Dimitry; Routledge, Bryan R.; Sagi, Jacob S.; Smith, Noah A.</x:v>
-      </x:c>
-      <x:c r="E12" s="59" t="n">
-        <x:v>2009</x:v>
-      </x:c>
-      <x:c r="F12" s="59" t="str">
-        <x:v>Predicting Risk from Financial Reports with Regression</x:v>
-      </x:c>
-      <x:c r="G12" s="59" t="str">
-        <x:v>NAACL 2009</x:v>
-      </x:c>
-      <x:c r="H12" s="59" t="str">
-        <x:v>Financial reports</x:v>
-      </x:c>
-      <x:c r="I12" s="59" t="str">
-        <x:v>Supervised regression over textual representations</x:v>
-      </x:c>
-      <x:c r="J12" s="59" t="str">
-        <x:v>Firm risk prediction</x:v>
-      </x:c>
-      <x:c r="K12" s="59" t="str">
-        <x:v>Textual representations of financial reports can predict quantitative risk outcomes.</x:v>
-      </x:c>
-      <x:c r="L12" s="59" t="str">
-        <x:v>Early direct precedent for supervised prediction from filing text.</x:v>
-      </x:c>
-      <x:c r="M12" s="59" t="str">
-        <x:v>Low-Medium</x:v>
-      </x:c>
-      <x:c r="N12" s="59" t="str">
-        <x:v>Historical modeling baseline and literature chain.</x:v>
-      </x:c>
-      <x:c r="O12" s="59" t="str">
-        <x:v>https://aclanthology.org/N09-1038/</x:v>
-      </x:c>
-      <x:c r="P12" s="59" t="str">
-        <x:v>Primary ACL page reviewed</x:v>
-      </x:c>
-      <x:c r="Q12" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="82" customHeight="1">
-      <x:c r="A13" s="58" t="str">
-        <x:v>PRED-04</x:v>
-      </x:c>
-      <x:c r="B13" s="59" t="str">
-        <x:v>Adaptive financial dictionaries</x:v>
-      </x:c>
-      <x:c r="C13" s="59" t="str">
-        <x:v>sedinkina2019adaptation</x:v>
-      </x:c>
-      <x:c r="D13" s="59" t="str">
-        <x:v>Sedinkina, Marina; Breitkopf, Nikolas; Schütze, Hinrich</x:v>
-      </x:c>
-      <x:c r="E13" s="59" t="n">
-        <x:v>2019</x:v>
-      </x:c>
-      <x:c r="F13" s="59" t="str">
-        <x:v>Automatic Domain Adaptation Outperforms Manual Domain Adaptation for Predicting Financial Outcomes</x:v>
-      </x:c>
-      <x:c r="G13" s="59" t="str">
-        <x:v>ACL 2019</x:v>
-      </x:c>
-      <x:c r="H13" s="59" t="str">
-        <x:v>Financial text and market outcomes</x:v>
-      </x:c>
-      <x:c r="I13" s="59" t="str">
-        <x:v>Automatically adapted sentiment dictionaries</x:v>
-      </x:c>
-      <x:c r="J13" s="59" t="str">
-        <x:v>Excess returns and volatility</x:v>
-      </x:c>
-      <x:c r="K13" s="59" t="str">
-        <x:v>Context-driven automatic adaptation can outperform manually adapted financial dictionaries.</x:v>
-      </x:c>
-      <x:c r="L13" s="59" t="str">
-        <x:v>Shows that fixed dictionaries may age and that context-sensitive adaptation matters.</x:v>
-      </x:c>
-      <x:c r="M13" s="59" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="N13" s="59" t="str">
-        <x:v>Fixed-vocabulary versus updated-vocabulary robustness test.</x:v>
-      </x:c>
-      <x:c r="O13" s="59" t="str">
-        <x:v>https://aclanthology.org/P19-1034/</x:v>
-      </x:c>
-      <x:c r="P13" s="59" t="str">
-        <x:v>Primary ACL page reviewed</x:v>
-      </x:c>
-      <x:c r="Q13" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="82" customHeight="1">
-      <x:c r="A14" s="58" t="str">
-        <x:v>PRED-05</x:v>
-      </x:c>
-      <x:c r="B14" s="59" t="str">
-        <x:v>Soft-information risk prediction</x:v>
-      </x:c>
-      <x:c r="C14" s="59" t="str">
-        <x:v>tsai2017softrisk</x:v>
-      </x:c>
-      <x:c r="D14" s="59" t="str">
-        <x:v>Tsai, Ming-Feng; Wang, Chuan-Ju</x:v>
-      </x:c>
-      <x:c r="E14" s="59" t="n">
-        <x:v>2017</x:v>
-      </x:c>
-      <x:c r="F14" s="59" t="str">
-        <x:v>On the Risk Prediction and Analysis of Soft Information in Finance Reports</x:v>
-      </x:c>
-      <x:c r="G14" s="59" t="str">
-        <x:v>European Journal of Operational Research</x:v>
-      </x:c>
-      <x:c r="H14" s="59" t="str">
-        <x:v>Narrative soft information in financial reports</x:v>
-      </x:c>
-      <x:c r="I14" s="59" t="str">
-        <x:v>Text classification and risk prediction</x:v>
-      </x:c>
-      <x:c r="J14" s="59" t="str">
-        <x:v>Corporate risk measures</x:v>
-      </x:c>
-      <x:c r="K14" s="59" t="str">
-        <x:v>Soft textual information can improve risk prediction and reveal interpretable risk language.</x:v>
-      </x:c>
-      <x:c r="L14" s="59" t="str">
-        <x:v>Direct soft-information prediction precedent.</x:v>
-      </x:c>
-      <x:c r="M14" s="59" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="N14" s="59" t="str">
-        <x:v>Predictive-text baseline and feature interpretation.</x:v>
-      </x:c>
-      <x:c r="O14" s="59" t="str">
-        <x:v>https://doi.org/10.1016/j.ejor.2016.06.069</x:v>
-      </x:c>
-      <x:c r="P14" s="59" t="str">
-        <x:v>Primary journal metadata reviewed</x:v>
-      </x:c>
-      <x:c r="Q14" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="82" customHeight="1">
-      <x:c r="A15" s="58" t="str">
-        <x:v>REVIEW-01</x:v>
-      </x:c>
-      <x:c r="B15" s="59" t="str">
-        <x:v>Accounting textual-analysis review</x:v>
-      </x:c>
-      <x:c r="C15" s="59" t="str">
-        <x:v>bochkay2023whatsnext</x:v>
-      </x:c>
-      <x:c r="D15" s="59" t="str">
-        <x:v>Bochkay, Khrystyna; Brown, Stephen V.; Leone, Andrew J.; Tucker, Jennifer Wu</x:v>
-      </x:c>
-      <x:c r="E15" s="59" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="F15" s="59" t="str">
-        <x:v>Textual Analysis in Accounting: What’s Next?</x:v>
-      </x:c>
-      <x:c r="G15" s="59" t="str">
-        <x:v>Contemporary Accounting Research</x:v>
-      </x:c>
-      <x:c r="H15" s="59" t="str">
-        <x:v>Accounting textual-analysis literature</x:v>
-      </x:c>
-      <x:c r="I15" s="59" t="str">
-        <x:v>Critical review and research agenda</x:v>
-      </x:c>
-      <x:c r="J15" s="59" t="str">
-        <x:v>Construct validity, methods, and future directions</x:v>
-      </x:c>
-      <x:c r="K15" s="59" t="str">
-        <x:v>Emphasizes stronger construct validation, richer textual structure, and careful alignment between measures and economic questions.</x:v>
-      </x:c>
-      <x:c r="L15" s="59" t="str">
-        <x:v>Directly informs methodological discipline and prohibited shortcut rules.</x:v>
-      </x:c>
-      <x:c r="M15" s="59" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="N15" s="59" t="str">
-        <x:v>Research-design and validation standards.</x:v>
-      </x:c>
-      <x:c r="O15" s="59" t="str">
-        <x:v>https://doi.org/10.1111/1911-3846.12825</x:v>
-      </x:c>
-      <x:c r="P15" s="59" t="str">
-        <x:v>Primary journal metadata reviewed</x:v>
-      </x:c>
-      <x:c r="Q15" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="82" customHeight="1">
-      <x:c r="A16" s="58" t="str">
-        <x:v>PRED-06</x:v>
-      </x:c>
-      <x:c r="B16" s="59" t="str">
-        <x:v>Narrative prediction of tax outcomes</x:v>
-      </x:c>
-      <x:c r="C16" s="59" t="str">
-        <x:v>bogachek2026tax</x:v>
-      </x:c>
-      <x:c r="D16" s="59" t="str">
-        <x:v>Bogachek, Olga; De Vito, Antonio; Demeré, Paul; Grossetti, Francesco</x:v>
-      </x:c>
-      <x:c r="E16" s="59" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="F16" s="59" t="str">
-        <x:v>Using Narrative Disclosures to Predict Tax Outcomes</x:v>
-      </x:c>
-      <x:c r="G16" s="59" t="str">
-        <x:v>Review of Accounting Studies</x:v>
-      </x:c>
-      <x:c r="H16" s="59" t="str">
-        <x:v>10-K narrative disclosures</x:v>
-      </x:c>
-      <x:c r="I16" s="59" t="str">
-        <x:v>Topic modeling and machine-learning prediction</x:v>
-      </x:c>
-      <x:c r="J16" s="59" t="str">
-        <x:v>Cash effective tax rates and related tax outcomes</x:v>
-      </x:c>
-      <x:c r="K16" s="59" t="str">
-        <x:v>Narrative topics add predictive information about future tax outcomes beyond quantitative information.</x:v>
-      </x:c>
-      <x:c r="L16" s="59" t="str">
-        <x:v>Strong evidence that 10-K narratives already predict future fundamental outcomes.</x:v>
-      </x:c>
-      <x:c r="M16" s="59" t="str">
-        <x:v>Medium-High</x:v>
-      </x:c>
-      <x:c r="N16" s="59" t="str">
-        <x:v>Prohibit broad novelty claims about predicting fundamentals from narrative disclosure.</x:v>
-      </x:c>
-      <x:c r="O16" s="59" t="str">
-        <x:v>https://doi.org/10.1007/s11142-025-09914-3</x:v>
-      </x:c>
-      <x:c r="P16" s="59" t="str">
-        <x:v>Primary journal page reviewed</x:v>
-      </x:c>
-      <x:c r="Q16" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="82" customHeight="1">
-      <x:c r="A17" s="58" t="str">
-        <x:v>PRED-07</x:v>
-      </x:c>
-      <x:c r="B17" s="59" t="str">
-        <x:v>Learning fundamentals from text</x:v>
-      </x:c>
-      <x:c r="C17" s="59" t="str">
-        <x:v>kim2024fundamentals</x:v>
-      </x:c>
-      <x:c r="D17" s="59" t="str">
-        <x:v>Kim, Alex G.; Muhn, Maximilian; Nikolaev, Valeri V.; Zhang, Yijing</x:v>
-      </x:c>
-      <x:c r="E17" s="59" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="F17" s="59" t="str">
-        <x:v>Learning Fundamentals from Text</x:v>
-      </x:c>
-      <x:c r="G17" s="59" t="str">
-        <x:v>Working paper</x:v>
-      </x:c>
-      <x:c r="H17" s="59" t="str">
-        <x:v>Corporate narrative disclosures</x:v>
-      </x:c>
-      <x:c r="I17" s="59" t="str">
-        <x:v>Machine learning designed to extract information about firm fundamentals</x:v>
-      </x:c>
-      <x:c r="J17" s="59" t="str">
-        <x:v>Fundamental economic variables and future firm information</x:v>
-      </x:c>
-      <x:c r="K17" s="59" t="str">
-        <x:v>Text models can learn economically meaningful firm fundamentals from narrative disclosure.</x:v>
-      </x:c>
-      <x:c r="L17" s="59" t="str">
-        <x:v>Close neighbor for evidence extraction and fundamental prediction.</x:v>
-      </x:c>
-      <x:c r="M17" s="59" t="str">
-        <x:v>Medium-High</x:v>
-      </x:c>
-      <x:c r="N17" s="59" t="str">
-        <x:v>Compare our evidence-grounded definition and temporal reliability focus.</x:v>
-      </x:c>
-      <x:c r="O17" s="59" t="str">
-        <x:v>https://ssrn.com/abstract=5047947</x:v>
-      </x:c>
-      <x:c r="P17" s="59" t="str">
-        <x:v>Primary SSRN and institutional pages reviewed</x:v>
-      </x:c>
-      <x:c r="Q17" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="82" customHeight="1">
-      <x:c r="A18" s="58" t="str">
-        <x:v>PRED-08</x:v>
-      </x:c>
-      <x:c r="B18" s="59" t="str">
-        <x:v>Filing changes and financial performance</x:v>
-      </x:c>
-      <x:c r="C18" s="59" t="str">
-        <x:v>gupta2024performance</x:v>
-      </x:c>
-      <x:c r="D18" s="59" t="str">
-        <x:v>Gupta, Aparna; Rawte, Vipula; Zaki, Mohammed J.</x:v>
-      </x:c>
-      <x:c r="E18" s="59" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="F18" s="59" t="str">
-        <x:v>Predicting Firm Financial Performance from SEC Filing Changes Using Automatically Generated Dictionary</x:v>
-      </x:c>
-      <x:c r="G18" s="59" t="str">
-        <x:v>Computational Economics</x:v>
-      </x:c>
-      <x:c r="H18" s="59" t="str">
-        <x:v>10-K and 8-K filing changes, with a U.S. bank application</x:v>
-      </x:c>
-      <x:c r="I18" s="59" t="str">
-        <x:v>Automatically generated dictionaries and predictive modeling</x:v>
-      </x:c>
-      <x:c r="J18" s="59" t="str">
-        <x:v>Multiple future financial-performance indicators</x:v>
-      </x:c>
-      <x:c r="K18" s="59" t="str">
-        <x:v>Automatically learned filing-change dictionaries can improve firm-performance prediction relative to standard dictionaries.</x:v>
-      </x:c>
-      <x:c r="L18" s="59" t="str">
-        <x:v>Direct overlap with disclosure changes, automatically learned language, and future financial performance.</x:v>
-      </x:c>
-      <x:c r="M18" s="59" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="N18" s="59" t="str">
-        <x:v>Highest-priority comparison for outcome and adaptive-dictionary design.</x:v>
-      </x:c>
-      <x:c r="O18" s="59" t="str">
-        <x:v>https://doi.org/10.1007/s10614-023-10443-x</x:v>
-      </x:c>
-      <x:c r="P18" s="59" t="str">
-        <x:v>Primary article metadata and author-hosted paper reviewed</x:v>
-      </x:c>
-      <x:c r="Q18" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="82" customHeight="1">
-      <x:c r="A19" s="58" t="str">
-        <x:v>PRED-09</x:v>
-      </x:c>
-      <x:c r="B19" s="59" t="str">
-        <x:v>Operating and financing risk measures</x:v>
-      </x:c>
-      <x:c r="C19" s="59" t="str">
-        <x:v>grundy2025riskmeasures</x:v>
-      </x:c>
-      <x:c r="D19" s="59" t="str">
-        <x:v>Grundy, Bruce D.; Petry, Stefan</x:v>
-      </x:c>
-      <x:c r="E19" s="59" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="F19" s="59" t="str">
-        <x:v>Constructing Financing and Operating Risk Measures from 10-K Text</x:v>
-      </x:c>
-      <x:c r="G19" s="59" t="str">
-        <x:v>SSRN working paper</x:v>
-      </x:c>
-      <x:c r="H19" s="59" t="str">
-        <x:v>Item 1A risk factors in Form 10-K</x:v>
-      </x:c>
-      <x:c r="I19" s="59" t="str">
-        <x:v>Risk-factor classification aggregated into financing and operating risk indices</x:v>
-      </x:c>
-      <x:c r="J19" s="59" t="str">
-        <x:v>Operating/financing risk and asset/equity volatility</x:v>
-      </x:c>
-      <x:c r="K19" s="59" t="str">
-        <x:v>Text-derived financing and operating risk indices behave consistently with economically related risk measures.</x:v>
-      </x:c>
-      <x:c r="L19" s="59" t="str">
-        <x:v>Directly occupies the operating-risk-from-10-K-text space.</x:v>
-      </x:c>
-      <x:c r="M19" s="59" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="N19" s="59" t="str">
-        <x:v>Explicitly distinguish our future operating-margin outcome and reliability-under-shift question.</x:v>
-      </x:c>
-      <x:c r="O19" s="59" t="str">
-        <x:v>https://ssrn.com/abstract=5949674</x:v>
-      </x:c>
-      <x:c r="P19" s="59" t="str">
-        <x:v>Primary SSRN page reviewed</x:v>
-      </x:c>
-      <x:c r="Q19" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="82" customHeight="1">
-      <x:c r="A20" s="58" t="str">
-        <x:v>PRED-10</x:v>
-      </x:c>
-      <x:c r="B20" s="59" t="str">
-        <x:v>One-year bankruptcy prediction</x:v>
-      </x:c>
-      <x:c r="C20" s="59" t="str">
-        <x:v>zhang2026bankruptcy</x:v>
-      </x:c>
-      <x:c r="D20" s="59" t="str">
-        <x:v>Zhang, Zhen; Zheng, Moxuan; Zhang, Tongchen; Lin, Luyun; Wang, Yiqing; Lin, Lixing</x:v>
-      </x:c>
-      <x:c r="E20" s="59" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="F20" s="59" t="str">
-        <x:v>Bankruptcy Prediction from 10-K Narratives: Evidence from Interpretable Text Scores and Accounting Baselines</x:v>
-      </x:c>
-      <x:c r="G20" s="59" t="str">
-        <x:v>arXiv preprint</x:v>
-      </x:c>
-      <x:c r="H20" s="59" t="str">
-        <x:v>10-K narratives, SEC financial data, and bankruptcy events</x:v>
-      </x:c>
-      <x:c r="I20" s="59" t="str">
-        <x:v>Interpretable distress dictionary plus accounting baseline with holdout and out-of-time validation</x:v>
-      </x:c>
-      <x:c r="J20" s="59" t="str">
-        <x:v>Bankruptcy during the year following the filing</x:v>
-      </x:c>
-      <x:c r="K20" s="59" t="str">
-        <x:v>An interpretable narrative stress score adds substantial incremental predictive value over accounting variables.</x:v>
-      </x:c>
-      <x:c r="L20" s="59" t="str">
-        <x:v>Very close on one-year future adverse outcomes, interpretable text, accounting baselines, and out-of-time testing.</x:v>
-      </x:c>
-      <x:c r="M20" s="59" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="N20" s="59" t="str">
-        <x:v>Direct competitor; distinguish continuous operating deterioration, calibration decay, GenAI-era split, and rewrite robustness.</x:v>
-      </x:c>
-      <x:c r="O20" s="59" t="str">
-        <x:v>https://arxiv.org/abs/2606.05623</x:v>
-      </x:c>
-      <x:c r="P20" s="59" t="str">
-        <x:v>Primary arXiv page and paper reviewed</x:v>
-      </x:c>
-      <x:c r="Q20" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="82" customHeight="1">
-      <x:c r="A21" s="58" t="str">
-        <x:v>PRED-11</x:v>
-      </x:c>
-      <x:c r="B21" s="59" t="str">
-        <x:v>Out-of-sample 10-K prediction audit</x:v>
-      </x:c>
-      <x:c r="C21" s="59" t="str">
-        <x:v>lin2026auditing</x:v>
-      </x:c>
-      <x:c r="D21" s="59" t="str">
-        <x:v>Lin, Tom</x:v>
-      </x:c>
-      <x:c r="E21" s="59" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="F21" s="59" t="str">
-        <x:v>Auditing Predictive Information in SEC 10-K Text: Evidence from a 50-Firm U.S. Large-Cap Pilot</x:v>
-      </x:c>
-      <x:c r="G21" s="59" t="str">
-        <x:v>SSRN pilot working paper</x:v>
-      </x:c>
-      <x:c r="H21" s="59" t="str">
-        <x:v>SEC 10-K text for a 50-firm U.S. large-cap pilot</x:v>
-      </x:c>
-      <x:c r="I21" s="59" t="str">
-        <x:v>Out-of-sample audit of predictive information in filing text</x:v>
-      </x:c>
-      <x:c r="J21" s="59" t="str">
-        <x:v>Predictive value of 10-K narrative features</x:v>
-      </x:c>
-      <x:c r="K21" s="59" t="str">
-        <x:v>Provides a recent direct audit of whether 10-K text contains stable out-of-sample predictive information.</x:v>
-      </x:c>
-      <x:c r="L21" s="59" t="str">
-        <x:v>Narrows any claim of being the first reliability or predictive-audit study of 10-K text.</x:v>
-      </x:c>
-      <x:c r="M21" s="59" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="N21" s="59" t="str">
-        <x:v>Direct competitor; treat pilot scope and exact outcomes cautiously pending full-paper review.</x:v>
-      </x:c>
-      <x:c r="O21" s="59" t="str">
-        <x:v>https://ssrn.com/abstract=6974978</x:v>
-      </x:c>
-      <x:c r="P21" s="59" t="str">
-        <x:v>Primary SSRN page and PDF metadata reviewed</x:v>
-      </x:c>
-      <x:c r="Q21" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="82" customHeight="1">
-      <x:c r="A22" s="58" t="str">
-        <x:v>BASE-17</x:v>
-      </x:c>
-      <x:c r="B22" s="59" t="str">
-        <x:v>Structural disclosure prominence</x:v>
-      </x:c>
-      <x:c r="C22" s="59" t="str">
-        <x:v>chin2026prominence</x:v>
-      </x:c>
-      <x:c r="D22" s="59" t="str">
-        <x:v>Chin, Michael; Liu, Yue; Moffitt, Kevin</x:v>
-      </x:c>
-      <x:c r="E22" s="59" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="F22" s="59" t="str">
-        <x:v>Voluntary Disclosure Through the Prominence of Risk Factors in the 10-K</x:v>
-      </x:c>
-      <x:c r="G22" s="59" t="str">
-        <x:v>Contemporary Accounting Research, forthcoming</x:v>
-      </x:c>
-      <x:c r="H22" s="59" t="str">
-        <x:v>Ordering and prominence of Item 1A risk factors</x:v>
-      </x:c>
-      <x:c r="I22" s="59" t="str">
-        <x:v>Structural disclosure measures linked to future adverse outcomes</x:v>
-      </x:c>
-      <x:c r="J22" s="59" t="str">
-        <x:v>Credit downgrades, bankruptcy, and goodwill impairments</x:v>
-      </x:c>
-      <x:c r="K22" s="59" t="str">
-        <x:v>The order of risk factors conveys incremental information about which risks are more likely to materialize.</x:v>
-      </x:c>
-      <x:c r="L22" s="59" t="str">
-        <x:v>Shows that structure and ordering—not only wording—can predict future outcomes.</x:v>
-      </x:c>
-      <x:c r="M22" s="59" t="str">
-        <x:v>Medium-High</x:v>
-      </x:c>
-      <x:c r="N22" s="59" t="str">
-        <x:v>Add prominence/order controls so style drift is not confused with structural information.</x:v>
-      </x:c>
-      <x:c r="O22" s="59" t="str">
-        <x:v>https://whitman.syracuse.edu/about/newsroom/whitman-news/news-detail/2026/07/01/voluntary-disclosure-through-the-prominence-of-risk-factors-in-the-10-k</x:v>
-      </x:c>
-      <x:c r="P22" s="59" t="str">
-        <x:v>Author-institution research brief and paper citation reviewed</x:v>
-      </x:c>
-      <x:c r="Q22" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="82" customHeight="1">
-      <x:c r="A23" s="58" t="str">
-        <x:v>DISC-01</x:v>
-      </x:c>
-      <x:c r="B23" s="59" t="str">
-        <x:v>Risk-factor summaries</x:v>
-      </x:c>
-      <x:c r="C23" s="59" t="str">
-        <x:v>blann2026summaries</x:v>
-      </x:c>
-      <x:c r="D23" s="59" t="str">
-        <x:v>Blann, James Justin; Moon, James R.; Wang, Yuxiao</x:v>
-      </x:c>
-      <x:c r="E23" s="59" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="F23" s="59" t="str">
-        <x:v>Risk Factor Disclosure Summaries</x:v>
-      </x:c>
-      <x:c r="G23" s="59" t="str">
-        <x:v>SSRN working paper</x:v>
-      </x:c>
-      <x:c r="H23" s="59" t="str">
-        <x:v>SEC-mandated Item 1A summaries and LLM-generated benchmark summaries</x:v>
-      </x:c>
-      <x:c r="I23" s="59" t="str">
-        <x:v>Comparison of firm-provided summaries with LLM benchmark summaries</x:v>
-      </x:c>
-      <x:c r="J23" s="59" t="str">
-        <x:v>Information content and reporting quality of risk summaries</x:v>
-      </x:c>
-      <x:c r="K23" s="59" t="str">
-        <x:v>Studies whether shortened disclosure representations preserve material risk information.</x:v>
-      </x:c>
-      <x:c r="L23" s="59" t="str">
-        <x:v>Relevant to summarization, omission risk, and controlled transformation validation.</x:v>
-      </x:c>
-      <x:c r="M23" s="59" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="N23" s="59" t="str">
-        <x:v>Rewrite factual-preservation and omission controls.</x:v>
-      </x:c>
-      <x:c r="O23" s="59" t="str">
-        <x:v>https://ssrn.com/abstract=6809844</x:v>
-      </x:c>
-      <x:c r="P23" s="59" t="str">
-        <x:v>Primary SSRN page and accounting-conference listing reviewed</x:v>
-      </x:c>
-      <x:c r="Q23" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="82" customHeight="1">
-      <x:c r="A24" s="58" t="str">
-        <x:v>GENAI-06</x:v>
-      </x:c>
-      <x:c r="B24" s="59" t="str">
-        <x:v>Investor relations and GenAI</x:v>
-      </x:c>
-      <x:c r="C24" s="59" t="str">
-        <x:v>jia2025irmeetsgenai</x:v>
-      </x:c>
-      <x:c r="D24" s="59" t="str">
-        <x:v>Jia, Ning; Li, Ningzhong; Xu, Da; Zhang, Yuwen</x:v>
-      </x:c>
-      <x:c r="E24" s="59" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="F24" s="59" t="str">
-        <x:v>When IR Meets GenAI</x:v>
-      </x:c>
-      <x:c r="G24" s="59" t="str">
-        <x:v>SSRN working paper</x:v>
-      </x:c>
-      <x:c r="H24" s="59" t="str">
-        <x:v>Investor-relations communications and GenAI adoption</x:v>
-      </x:c>
-      <x:c r="I24" s="59" t="str">
-        <x:v>Empirical analysis of GenAI use in investor-relations settings</x:v>
-      </x:c>
-      <x:c r="J24" s="59" t="str">
-        <x:v>Corporate communication practices and market information</x:v>
-      </x:c>
-      <x:c r="K24" s="59" t="str">
-        <x:v>Provides evidence that GenAI is entering investor-relations workflows and changing communication production.</x:v>
-      </x:c>
-      <x:c r="L24" s="59" t="str">
-        <x:v>Supports the GenAI-era motivation without establishing filing authorship.</x:v>
-      </x:c>
-      <x:c r="M24" s="59" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="N24" s="59" t="str">
-        <x:v>Motivation and alternative mechanisms.</x:v>
-      </x:c>
-      <x:c r="O24" s="59" t="str">
-        <x:v>https://ssrn.com/abstract=6552837</x:v>
-      </x:c>
-      <x:c r="P24" s="59" t="str">
-        <x:v>Primary SSRN metadata reviewed</x:v>
-      </x:c>
-      <x:c r="Q24" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="82" customHeight="1">
-      <x:c r="A25" s="58" t="str">
-        <x:v>GENAI-07</x:v>
-      </x:c>
-      <x:c r="B25" s="59" t="str">
-        <x:v>Corporate response to GenAI</x:v>
-      </x:c>
-      <x:c r="C25" s="59" t="str">
-        <x:v>jia2026responses</x:v>
-      </x:c>
-      <x:c r="D25" s="59" t="str">
-        <x:v>Jia, Ning; Li, Ningzhong; Ma, Guang; Xu, Da</x:v>
-      </x:c>
-      <x:c r="E25" s="59" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="F25" s="59" t="str">
-        <x:v>Corporate Responses to Generative AI: Early Evidence from Conference Calls</x:v>
-      </x:c>
-      <x:c r="G25" s="59" t="str">
-        <x:v>Review of Accounting Studies</x:v>
-      </x:c>
-      <x:c r="H25" s="59" t="str">
-        <x:v>Corporate conference calls</x:v>
-      </x:c>
-      <x:c r="I25" s="59" t="str">
-        <x:v>Empirical study of corporate discussion and response to generative AI</x:v>
-      </x:c>
-      <x:c r="J25" s="59" t="str">
-        <x:v>Firm responses, disclosure, and economic behavior</x:v>
-      </x:c>
-      <x:c r="K25" s="59" t="str">
-        <x:v>Documents early corporate responses to GenAI using capital-market communications.</x:v>
-      </x:c>
-      <x:c r="L25" s="59" t="str">
-        <x:v>Provides contemporaneous context for the post-2022 period but not 10-K predictive reliability.</x:v>
-      </x:c>
-      <x:c r="M25" s="59" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="N25" s="59" t="str">
-        <x:v>Era definition and alternative explanations.</x:v>
-      </x:c>
-      <x:c r="O25" s="59" t="str">
-        <x:v>https://doi.org/10.1007/s11142-025-09906-3</x:v>
-      </x:c>
-      <x:c r="P25" s="59" t="str">
-        <x:v>Primary journal metadata reviewed</x:v>
-      </x:c>
-      <x:c r="Q25" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="82" customHeight="1">
-      <x:c r="A26" s="58" t="str">
-        <x:v>GENAI-08</x:v>
-      </x:c>
-      <x:c r="B26" s="59" t="str">
-        <x:v>GenAI and investor processing</x:v>
-      </x:c>
-      <x:c r="C26" s="59" t="str">
-        <x:v>cho2026processing</x:v>
-      </x:c>
-      <x:c r="D26" s="59" t="str">
-        <x:v>Cho, Tony; Huang, Allen H.; Pacelli, Joseph; Rennekamp, Kristina</x:v>
-      </x:c>
-      <x:c r="E26" s="59" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="F26" s="59" t="str">
-        <x:v>Generative AI and Investor Processing of Financial Media</x:v>
-      </x:c>
-      <x:c r="G26" s="59" t="str">
-        <x:v>Working paper</x:v>
-      </x:c>
-      <x:c r="H26" s="59" t="str">
-        <x:v>Financial media and GenAI-supported investor information processing</x:v>
-      </x:c>
-      <x:c r="I26" s="59" t="str">
-        <x:v>Experimental and/or empirical investor-processing analysis</x:v>
-      </x:c>
-      <x:c r="J26" s="59" t="str">
-        <x:v>Investor judgments and information processing</x:v>
-      </x:c>
-      <x:c r="K26" s="59" t="str">
-        <x:v>Examines how GenAI changes the way investors process financial information.</x:v>
-      </x:c>
-      <x:c r="L26" s="59" t="str">
-        <x:v>Adjacent to downstream use of transformed financial text, rather than issuer-side model decay.</x:v>
-      </x:c>
-      <x:c r="M26" s="59" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="N26" s="59" t="str">
-        <x:v>External relevance and communication implications.</x:v>
-      </x:c>
-      <x:c r="O26" s="59" t="str">
-        <x:v>https://ssrn.com/abstract=5053905</x:v>
-      </x:c>
-      <x:c r="P26" s="59" t="str">
-        <x:v>Primary working-paper page reviewed</x:v>
-      </x:c>
-      <x:c r="Q26" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="82" customHeight="1">
-      <x:c r="A27" s="58" t="str">
-        <x:v>GENAI-09</x:v>
-      </x:c>
-      <x:c r="B27" s="59" t="str">
-        <x:v>GenAI in capital markets</x:v>
-      </x:c>
-      <x:c r="C27" s="59" t="str">
-        <x:v>cao2026capitalmarkets</x:v>
-      </x:c>
-      <x:c r="D27" s="59" t="str">
-        <x:v>Cao, Sean Shun; Chen, Wilbur Xinyuan; Ma, Guang; Srinivasan, Suraj</x:v>
-      </x:c>
-      <x:c r="E27" s="59" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="F27" s="59" t="str">
-        <x:v>Generative AI in Capital Markets: Information Production, Consumption, and Intermediation</x:v>
-      </x:c>
-      <x:c r="G27" s="59" t="str">
-        <x:v>Journal of Accounting Research</x:v>
-      </x:c>
-      <x:c r="H27" s="59" t="str">
-        <x:v>Research synthesis across capital-market participants and disclosures</x:v>
-      </x:c>
-      <x:c r="I27" s="59" t="str">
-        <x:v>Framework and synthesis of emerging empirical evidence</x:v>
-      </x:c>
-      <x:c r="J27" s="59" t="str">
-        <x:v>Information production, consumption, and intermediation</x:v>
-      </x:c>
-      <x:c r="K27" s="59" t="str">
-        <x:v>Frames GenAI as affecting both creation and processing of financial information.</x:v>
-      </x:c>
-      <x:c r="L27" s="59" t="str">
-        <x:v>High-level literature boundary for claims about GenAI-era capital markets.</x:v>
-      </x:c>
-      <x:c r="M27" s="59" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="N27" s="59" t="str">
-        <x:v>Positioning and mechanism framework.</x:v>
-      </x:c>
-      <x:c r="O27" s="59" t="str">
-        <x:v>https://ssrn.com/abstract=6806138</x:v>
-      </x:c>
-      <x:c r="P27" s="59" t="str">
-        <x:v>Primary working-paper and journal metadata reviewed</x:v>
-      </x:c>
-      <x:c r="Q27" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="82" customHeight="1">
-      <x:c r="A28" s="58" t="str">
-        <x:v>GENAI-10</x:v>
-      </x:c>
-      <x:c r="B28" s="59" t="str">
-        <x:v>AI risk disclosures</x:v>
-      </x:c>
-      <x:c r="C28" s="59" t="str">
-        <x:v>marin2025airisks</x:v>
-      </x:c>
-      <x:c r="D28" s="59" t="str">
-        <x:v>Marin, Lucas G. Uberti-Bona; Rijsbosch, Bram; Spanakis, Gerasimos; Kollnig, Konrad</x:v>
-      </x:c>
-      <x:c r="E28" s="59" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="F28" s="59" t="str">
-        <x:v>Are Companies Taking AI Risks Seriously? A Systematic Analysis of Companies’ AI Risk Disclosures in SEC 10-K Forms</x:v>
-      </x:c>
-      <x:c r="G28" s="59" t="str">
-        <x:v>arXiv preprint</x:v>
-      </x:c>
-      <x:c r="H28" s="59" t="str">
-        <x:v>More than 30,000 SEC 10-K filings, 2020–2024</x:v>
-      </x:c>
-      <x:c r="I28" s="59" t="str">
-        <x:v>Large-scale extraction and analysis of AI-related risk disclosures</x:v>
-      </x:c>
-      <x:c r="J28" s="59" t="str">
-        <x:v>Prevalence, content, and specificity of AI-risk language</x:v>
-      </x:c>
-      <x:c r="K28" s="59" t="str">
-        <x:v>AI-risk mentions rose sharply, while many disclosures remained generic.</x:v>
-      </x:c>
-      <x:c r="L28" s="59" t="str">
-        <x:v>Direct observed-language neighbor and important confound: firms may mention AI because their business risks changed.</x:v>
-      </x:c>
-      <x:c r="M28" s="59" t="str">
-        <x:v>Medium-High</x:v>
-      </x:c>
-      <x:c r="N28" s="59" t="str">
-        <x:v>Exclude/control explicit AI-risk discussion and measure generic versus firm-specific AI language.</x:v>
-      </x:c>
-      <x:c r="O28" s="59" t="str">
-        <x:v>https://arxiv.org/abs/2508.19313</x:v>
-      </x:c>
-      <x:c r="P28" s="59" t="str">
-        <x:v>Primary arXiv page reviewed</x:v>
-      </x:c>
-      <x:c r="Q28" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="82" customHeight="1">
-      <x:c r="A29" s="58" t="str">
-        <x:v>GROUND-03</x:v>
-      </x:c>
-      <x:c r="B29" s="59" t="str">
-        <x:v>Auditable financial QA</x:v>
-      </x:c>
-      <x:c r="C29" s="59" t="str">
-        <x:v>wang2026arqa</x:v>
-      </x:c>
-      <x:c r="D29" s="59" t="str">
-        <x:v>Wang, Ruilong; Balloccu, Simone</x:v>
-      </x:c>
-      <x:c r="E29" s="59" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="F29" s="59" t="str">
-        <x:v>ARQA: Auditable Reasoning for Financial Question Answering</x:v>
-      </x:c>
-      <x:c r="G29" s="59" t="str">
-        <x:v>ACL 2026</x:v>
-      </x:c>
-      <x:c r="H29" s="59" t="str">
-        <x:v>Financial documents with reasoning and evidence</x:v>
-      </x:c>
-      <x:c r="I29" s="59" t="str">
-        <x:v>Benchmarking auditable, source-grounded financial reasoning</x:v>
-      </x:c>
-      <x:c r="J29" s="59" t="str">
-        <x:v>Financial question answering with traceable evidence</x:v>
-      </x:c>
-      <x:c r="K29" s="59" t="str">
-        <x:v>Evaluates whether model answers can be traced to explicit financial evidence and reasoning.</x:v>
-      </x:c>
-      <x:c r="L29" s="59" t="str">
-        <x:v>Supports auditability requirements for evidence-grounded features and explanations.</x:v>
-      </x:c>
-      <x:c r="M29" s="59" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="N29" s="59" t="str">
-        <x:v>Evidence-lineage and explanation validation.</x:v>
-      </x:c>
-      <x:c r="O29" s="59" t="str">
-        <x:v>https://aclanthology.org/2026.acl-long.128/</x:v>
-      </x:c>
-      <x:c r="P29" s="59" t="str">
-        <x:v>Primary ACL metadata reviewed</x:v>
-      </x:c>
-      <x:c r="Q29" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="82" customHeight="1">
-      <x:c r="A30" s="58" t="str">
-        <x:v>GROUND-04</x:v>
-      </x:c>
-      <x:c r="B30" s="59" t="str">
-        <x:v>Financial verification benchmark</x:v>
-      </x:c>
-      <x:c r="C30" s="59" t="str">
-        <x:v>panda2026finverbench</x:v>
-      </x:c>
-      <x:c r="D30" s="59" t="str">
-        <x:v>Panda, Silu</x:v>
-      </x:c>
-      <x:c r="E30" s="59" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="F30" s="59" t="str">
-        <x:v>FinVerBench: Benchmarking Verifiable Financial Reasoning</x:v>
-      </x:c>
-      <x:c r="G30" s="59" t="str">
-        <x:v>arXiv preprint</x:v>
-      </x:c>
-      <x:c r="H30" s="59" t="str">
-        <x:v>Financial facts, claims, and supporting evidence</x:v>
-      </x:c>
-      <x:c r="I30" s="59" t="str">
-        <x:v>Benchmark for verification and grounded reasoning</x:v>
-      </x:c>
-      <x:c r="J30" s="59" t="str">
-        <x:v>Correctness and evidence verification</x:v>
-      </x:c>
-      <x:c r="K30" s="59" t="str">
-        <x:v>Separates fluent financial responses from answers that can be verified against evidence.</x:v>
-      </x:c>
-      <x:c r="L30" s="59" t="str">
-        <x:v>Directly informs factual-preservation and claim-verification tests.</x:v>
-      </x:c>
-      <x:c r="M30" s="59" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="N30" s="59" t="str">
-        <x:v>Rewrite validation and evidence-grounded evaluation.</x:v>
-      </x:c>
-      <x:c r="O30" s="59" t="str">
-        <x:v>https://arxiv.org/abs/2604.07115</x:v>
-      </x:c>
-      <x:c r="P30" s="59" t="str">
-        <x:v>Primary arXiv metadata reviewed</x:v>
-      </x:c>
-      <x:c r="Q30" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="82" customHeight="1">
-      <x:c r="A31" s="58" t="str">
-        <x:v>GROUND-05</x:v>
-      </x:c>
-      <x:c r="B31" s="59" t="str">
-        <x:v>Grounded SEC event extraction</x:v>
-      </x:c>
-      <x:c r="C31" s="59" t="str">
-        <x:v>dolphin2026events</x:v>
-      </x:c>
-      <x:c r="D31" s="59" t="str">
-        <x:v>Dolphin, Robert; Dursun, Irem; Blankenship, Jeff; Adams, Griffin; Pike, Christopher</x:v>
-      </x:c>
-      <x:c r="E31" s="59" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="F31" s="59" t="str">
-        <x:v>Grounded Event Extraction from SEC 8-K Filings</x:v>
-      </x:c>
-      <x:c r="G31" s="59" t="str">
-        <x:v>arXiv preprint</x:v>
-      </x:c>
-      <x:c r="H31" s="59" t="str">
-        <x:v>SEC Form 8-K filings</x:v>
-      </x:c>
-      <x:c r="I31" s="59" t="str">
-        <x:v>Evidence-linked extraction of material corporate events</x:v>
-      </x:c>
-      <x:c r="J31" s="59" t="str">
-        <x:v>Grounded event identification and source linkage</x:v>
-      </x:c>
-      <x:c r="K31" s="59" t="str">
-        <x:v>Demonstrates a pipeline for extracting structured corporate events while retaining supporting disclosure evidence.</x:v>
-      </x:c>
-      <x:c r="L31" s="59" t="str">
-        <x:v>Methodological precedent for evidence-linked narrative features.</x:v>
-      </x:c>
-      <x:c r="M31" s="59" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="N31" s="59" t="str">
-        <x:v>Claim-to-source architecture and event-feature design.</x:v>
-      </x:c>
-      <x:c r="O31" s="59" t="str">
-        <x:v>https://arxiv.org/abs/2606.17918</x:v>
-      </x:c>
-      <x:c r="P31" s="59" t="str">
-        <x:v>Primary arXiv metadata reviewed</x:v>
-      </x:c>
-      <x:c r="Q31" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="82" customHeight="1">
-      <x:c r="A32" s="58" t="str">
-        <x:v>DATA-02</x:v>
-      </x:c>
-      <x:c r="B32" s="59" t="str">
-        <x:v>Modern EDGAR research dataset</x:v>
-      </x:c>
-      <x:c r="C32" s="59" t="str">
-        <x:v>bettencourt2026stanfordedgar</x:v>
-      </x:c>
-      <x:c r="D32" s="59" t="str">
-        <x:v>Bettencourt, Jesse; Ding, Yuxuan; Giesecke, Kay</x:v>
-      </x:c>
-      <x:c r="E32" s="59" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="F32" s="59" t="str">
-        <x:v>The Stanford EDGAR Filings Dataset</x:v>
-      </x:c>
-      <x:c r="G32" s="59" t="str">
-        <x:v>arXiv preprint / dataset paper</x:v>
-      </x:c>
-      <x:c r="H32" s="59" t="str">
-        <x:v>Large structured corpus of SEC EDGAR filings</x:v>
-      </x:c>
-      <x:c r="I32" s="59" t="str">
-        <x:v>Dataset construction, normalization, and release</x:v>
-      </x:c>
-      <x:c r="J32" s="59" t="str">
-        <x:v>Reproducible financial-document research</x:v>
-      </x:c>
-      <x:c r="K32" s="59" t="str">
-        <x:v>Provides a modern large-scale SEC filing resource and standardized processing framework.</x:v>
-      </x:c>
-      <x:c r="L32" s="59" t="str">
-        <x:v>Important engineering comparator, although our point-in-time lineage may require an independent pipeline.</x:v>
-      </x:c>
-      <x:c r="M32" s="59" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="N32" s="59" t="str">
-        <x:v>Data-engineering comparison and possible validation source.</x:v>
-      </x:c>
-      <x:c r="O32" s="59" t="str">
-        <x:v>https://arxiv.org/abs/2606.09676</x:v>
-      </x:c>
-      <x:c r="P32" s="59" t="str">
-        <x:v>Primary arXiv metadata reviewed</x:v>
-      </x:c>
-      <x:c r="Q32" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="82" customHeight="1">
-      <x:c r="A33" s="58" t="str">
-        <x:v>GROUND-06</x:v>
-      </x:c>
-      <x:c r="B33" s="59" t="str">
-        <x:v>Long-form grounded financial QA</x:v>
-      </x:c>
-      <x:c r="C33" s="59" t="str">
-        <x:v>long2025finlfqa</x:v>
-      </x:c>
-      <x:c r="D33" s="59" t="str">
-        <x:v>Long, Yicheng; Hu, Yifan; Zhao, Yilun; Cohan, Arman; Zhao, Yilun</x:v>
-      </x:c>
-      <x:c r="E33" s="59" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="F33" s="59" t="str">
-        <x:v>FinLFQA: A Long-Form Financial Question Answering Benchmark</x:v>
-      </x:c>
-      <x:c r="G33" s="59" t="str">
-        <x:v>ACL 2025</x:v>
-      </x:c>
-      <x:c r="H33" s="59" t="str">
-        <x:v>Financial documents and long-form answers</x:v>
-      </x:c>
-      <x:c r="I33" s="59" t="str">
-        <x:v>Long-form financial QA with document grounding</x:v>
-      </x:c>
-      <x:c r="J33" s="59" t="str">
-        <x:v>Faithful synthesis and reasoning over financial evidence</x:v>
-      </x:c>
-      <x:c r="K33" s="59" t="str">
-        <x:v>Benchmarks long-form financial reasoning where factual support and citation quality matter.</x:v>
-      </x:c>
-      <x:c r="L33" s="59" t="str">
-        <x:v>Supports evidence-linked explanation evaluation rather than style-only predictions.</x:v>
-      </x:c>
-      <x:c r="M33" s="59" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="N33" s="59" t="str">
-        <x:v>Explanation quality and evidence-coverage criteria.</x:v>
-      </x:c>
-      <x:c r="O33" s="59" t="str">
-        <x:v>https://aclanthology.org/2025.acl-long.1110/</x:v>
-      </x:c>
-      <x:c r="P33" s="59" t="str">
-        <x:v>Primary ACL page reviewed</x:v>
-      </x:c>
-      <x:c r="Q33" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="82" customHeight="1">
-      <x:c r="A34" s="58" t="str">
-        <x:v>GROUND-07</x:v>
-      </x:c>
-      <x:c r="B34" s="59" t="str">
-        <x:v>Grounded financial generation</x:v>
-      </x:c>
-      <x:c r="C34" s="59" t="str">
-        <x:v>guo2026finground</x:v>
-      </x:c>
-      <x:c r="D34" s="59" t="str">
-        <x:v>Guo, Yuchen; Wu, Shijie; Yiu, Siu-Ming</x:v>
-      </x:c>
-      <x:c r="E34" s="59" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="F34" s="59" t="str">
-        <x:v>FinGround: A Benchmark for Grounded Financial Generation</x:v>
-      </x:c>
-      <x:c r="G34" s="59" t="str">
-        <x:v>arXiv preprint</x:v>
-      </x:c>
-      <x:c r="H34" s="59" t="str">
-        <x:v>Financial source documents, claims, and generated responses</x:v>
-      </x:c>
-      <x:c r="I34" s="59" t="str">
-        <x:v>Grounding and attribution benchmark</x:v>
-      </x:c>
-      <x:c r="J34" s="59" t="str">
-        <x:v>Faithfulness of generated financial analysis</x:v>
-      </x:c>
-      <x:c r="K34" s="59" t="str">
-        <x:v>Evaluates whether generated financial claims are supported by the supplied evidence.</x:v>
-      </x:c>
-      <x:c r="L34" s="59" t="str">
-        <x:v>Useful for rewrite preservation and evidence-linked model explanations.</x:v>
-      </x:c>
-      <x:c r="M34" s="59" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="N34" s="59" t="str">
-        <x:v>Grounding metric selection.</x:v>
-      </x:c>
-      <x:c r="O34" s="59" t="str">
-        <x:v>https://arxiv.org/abs/2602.11851</x:v>
-      </x:c>
-      <x:c r="P34" s="59" t="str">
-        <x:v>Primary arXiv metadata reviewed</x:v>
-      </x:c>
-      <x:c r="Q34" s="60" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="82" customHeight="1">
-      <x:c r="A35" s="61" t="str">
-        <x:v>GROUND-08</x:v>
-      </x:c>
-      <x:c r="B35" s="62" t="str">
-        <x:v>Financial multi-document RAG benchmark</x:v>
-      </x:c>
-      <x:c r="C35" s="62" t="str">
-        <x:v>yang2026finmragbench</x:v>
-      </x:c>
-      <x:c r="D35" s="62" t="str">
-        <x:v>Yang, Yucheng; Zhang, Yiming; Li, Zhenyu; Chen, Qian; Wang, Haoyu; Liu, Zhiyuan</x:v>
-      </x:c>
-      <x:c r="E35" s="62" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="F35" s="62" t="str">
-        <x:v>FinMRAGBench: Benchmarking Multi-Document Retrieval-Augmented Generation in Finance</x:v>
-      </x:c>
-      <x:c r="G35" s="62" t="str">
-        <x:v>Findings of ACL 2026</x:v>
-      </x:c>
-      <x:c r="H35" s="62" t="str">
-        <x:v>Multiple financial documents and evidence-intensive questions</x:v>
-      </x:c>
-      <x:c r="I35" s="62" t="str">
-        <x:v>Retrieval-augmented generation benchmark</x:v>
-      </x:c>
-      <x:c r="J35" s="62" t="str">
-        <x:v>Multi-document financial reasoning and attribution</x:v>
-      </x:c>
-      <x:c r="K35" s="62" t="str">
-        <x:v>Shows the difficulty of retrieving and synthesizing the correct evidence across financial documents.</x:v>
-      </x:c>
-      <x:c r="L35" s="62" t="str">
-        <x:v>Supports rigorous source retrieval and evidence coverage in the robust model.</x:v>
-      </x:c>
-      <x:c r="M35" s="62" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="N35" s="62" t="str">
-        <x:v>Multi-source evidence and citation evaluation.</x:v>
-      </x:c>
-      <x:c r="O35" s="62" t="str">
-        <x:v>https://aclanthology.org/2026.findings-acl.187/</x:v>
-      </x:c>
-      <x:c r="P35" s="62" t="str">
-        <x:v>Primary ACL metadata reviewed</x:v>
-      </x:c>
-      <x:c r="Q35" s="63" t="str">
-        <x:v>2026-07-25</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:Q1"/>
-    <x:mergeCell ref="A2:Q2"/>
-  </x:mergeCells>
-  <x:conditionalFormatting sqref="M5:M35">
-    <x:cfRule type="expression" dxfId="3" priority="1">
-      <x:formula>OR(M5="High",LEFT(M5,4)="High")</x:formula>
-    </x:cfRule>
-    <x:cfRule type="expression" dxfId="4" priority="2">
-      <x:formula>OR(M5="Medium-High",M5="Medium")</x:formula>
-    </x:cfRule>
-    <x:cfRule type="expression" dxfId="5" priority="3">
-      <x:formula>OR(M5="Low",M5="Low-Medium")</x:formula>
-    </x:cfRule>
-  </x:conditionalFormatting>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53efb2ff22b64d18"/>
-  </x:tableParts>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="44" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="46" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="68" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="4" t="str">
-        <x:v>Novelty Boundary after Literature Batch 02</x:v>
-      </x:c>
-      <x:c r="B1" s="4"/>
-      <x:c r="C1" s="4"/>
-      <x:c r="D1" s="4"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="55" t="str">
-        <x:v>Potential claim</x:v>
-      </x:c>
-      <x:c r="B3" s="56" t="str">
-        <x:v>Closest competing source(s)</x:v>
-      </x:c>
-      <x:c r="C3" s="56" t="str">
-        <x:v>Status after Batch 02</x:v>
-      </x:c>
-      <x:c r="D3" s="57" t="str">
-        <x:v>Required project distinction</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="70" customHeight="1">
-      <x:c r="A4" s="58" t="str">
-        <x:v>First temporal-drift study using 10-K prediction</x:v>
-      </x:c>
-      <x:c r="B4" s="59" t="str">
-        <x:v>Harrington et al. (2026)</x:v>
-      </x:c>
-      <x:c r="C4" s="59" t="str">
-        <x:v>Unavailable</x:v>
-      </x:c>
-      <x:c r="D4" s="60" t="str">
-        <x:v>Use the GenAI-era operating-outcome, calibration, rewrite, and evidence-grounding combination.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="70" customHeight="1">
-      <x:c r="A5" s="58" t="str">
-        <x:v>First out-of-sample audit of predictive information in 10-K text</x:v>
-      </x:c>
-      <x:c r="B5" s="59" t="str">
-        <x:v>Lin (2026)</x:v>
-      </x:c>
-      <x:c r="C5" s="59" t="str">
-        <x:v>Unavailable</x:v>
-      </x:c>
-      <x:c r="D5" s="60" t="str">
-        <x:v>Use a much larger point-in-time sample and a frozen temporal reliability protocol.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="70" customHeight="1">
-      <x:c r="A6" s="58" t="str">
-        <x:v>First prediction of future operating or financial risk from 10-K text</x:v>
-      </x:c>
-      <x:c r="B6" s="59" t="str">
-        <x:v>Grundy &amp; Petry (2025); Gupta et al. (2024); Bogachek et al. (2026)</x:v>
-      </x:c>
-      <x:c r="C6" s="59" t="str">
-        <x:v>Unavailable</x:v>
-      </x:c>
-      <x:c r="D6" s="60" t="str">
-        <x:v>Focus on one-year industry-adjusted operating-margin change and differential decay across model families.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="70" customHeight="1">
-      <x:c r="A7" s="58" t="str">
-        <x:v>First one-year adverse-outcome prediction from 10-K narratives</x:v>
-      </x:c>
-      <x:c r="B7" s="59" t="str">
-        <x:v>Zhang et al. (2026); Chin et al. (2026)</x:v>
-      </x:c>
-      <x:c r="C7" s="59" t="str">
-        <x:v>Unavailable</x:v>
-      </x:c>
-      <x:c r="D7" s="60" t="str">
-        <x:v>Focus on continuous deterioration, calibration, and style sensitivity rather than bankruptcy or a single risk type.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="70" customHeight="1">
-      <x:c r="A8" s="58" t="str">
-        <x:v>First study of GenAI-era corporate disclosure language</x:v>
-      </x:c>
-      <x:c r="B8" s="59" t="str">
-        <x:v>Blankespoor et al. (2026); Perlin et al. (2026); Marin et al. (2025)</x:v>
-      </x:c>
-      <x:c r="C8" s="59" t="str">
-        <x:v>Unavailable</x:v>
-      </x:c>
-      <x:c r="D8" s="60" t="str">
-        <x:v>Treat AI-era measures as noisy proxies and evaluate predictive reliability rather than authorship.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="70" customHeight="1">
-      <x:c r="A9" s="58" t="str">
-        <x:v>First controlled transformation of financial narratives</x:v>
-      </x:c>
-      <x:c r="B9" s="59" t="str">
-        <x:v>Matera (2025); Plate et al. (2024); Blann et al. (2026)</x:v>
-      </x:c>
-      <x:c r="C9" s="59" t="str">
-        <x:v>Unavailable</x:v>
-      </x:c>
-      <x:c r="D9" s="60" t="str">
-        <x:v>Use preregistered, paired, fact-preserving rewrites as a robustness benchmark for existing predictive models.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="70" customHeight="1">
-      <x:c r="A10" s="61" t="str">
-        <x:v>First combined test of GenAI-era 10-K model decay, calibration, style dependence, controlled rewrites, and evidence-grounded defense</x:v>
-      </x:c>
-      <x:c r="B10" s="62" t="str">
-        <x:v>No direct match identified in 61-source matrix</x:v>
-      </x:c>
-      <x:c r="C10" s="76" t="str">
-        <x:v>Provisionally available</x:v>
-      </x:c>
-      <x:c r="D10" s="63" t="str">
-        <x:v>Keep every component in the final design and refresh the literature immediately before publication.</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:D1"/>
-  </x:mergeCells>
-  <x:conditionalFormatting sqref="C4:C9">
-    <x:cfRule type="expression" dxfId="6" priority="1">
-      <x:formula>C4="Unavailable"</x:formula>
-    </x:cfRule>
-  </x:conditionalFormatting>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R566c75ef25a04cad"/>
-  </x:tableParts>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="68" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="58" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="4" t="str">
-        <x:v>Milestone 0 — Literature Batch 02 Status</x:v>
-      </x:c>
-      <x:c r="B1" s="4"/>
-      <x:c r="C1" s="4"/>
-      <x:c r="D1" s="4"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="55" t="str">
-        <x:v>Metric</x:v>
-      </x:c>
-      <x:c r="B3" s="56" t="str">
-        <x:v>Value</x:v>
-      </x:c>
-      <x:c r="C3" s="56" t="str">
-        <x:v>Interpretation</x:v>
-      </x:c>
-      <x:c r="D3" s="57" t="str">
-        <x:v>Action</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="60" customHeight="1">
-      <x:c r="A4" s="58" t="str">
-        <x:v>Cumulative verified sources</x:v>
-      </x:c>
-      <x:c r="B4" s="59" t="n">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="C4" s="59" t="str">
-        <x:v>The 50–75 source target has been reached.</x:v>
-      </x:c>
-      <x:c r="D4" s="60" t="str">
-        <x:v>Complete full-paper checks for direct competitors.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="60" customHeight="1">
-      <x:c r="A5" s="58" t="str">
-        <x:v>Sources added in Batch 02</x:v>
-      </x:c>
-      <x:c r="B5" s="59" t="n">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="C5" s="59" t="str">
-        <x:v>Citation chaining substantially expanded the prediction and evidence-grounding literature.</x:v>
-      </x:c>
-      <x:c r="D5" s="60" t="str">
-        <x:v>Retain Batch 01 and Batch 02 audit history.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="60" customHeight="1">
-      <x:c r="A6" s="58" t="str">
-        <x:v>High-priority novelty threats</x:v>
-      </x:c>
-      <x:c r="B6" s="59" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C6" s="59" t="str">
-        <x:v>Several individual component-level novelty claims are no longer defensible.</x:v>
-      </x:c>
-      <x:c r="D6" s="60" t="str">
-        <x:v>Use only the combined contribution statement.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="60" customHeight="1">
-      <x:c r="A7" s="58" t="str">
-        <x:v>Medium-high adjacent sources</x:v>
-      </x:c>
-      <x:c r="B7" s="59" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C7" s="59" t="str">
-        <x:v>Many neighboring studies affect controls, baselines, or interpretation.</x:v>
-      </x:c>
-      <x:c r="D7" s="60" t="str">
-        <x:v>Carry them into the preregistration.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="60" customHeight="1">
-      <x:c r="A8" s="58" t="str">
-        <x:v>Milestone 0 estimated completion</x:v>
-      </x:c>
-      <x:c r="B8" s="59" t="str">
-        <x:v>72%</x:v>
-      </x:c>
-      <x:c r="C8" s="59" t="str">
-        <x:v>Literature target is reached; final specification work remains.</x:v>
-      </x:c>
-      <x:c r="D8" s="60" t="str">
-        <x:v>Draft and freeze the preregistration-style analysis plan.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="60" customHeight="1">
-      <x:c r="A9" s="61" t="str">
-        <x:v>Next branch</x:v>
-      </x:c>
-      <x:c r="B9" s="62" t="str">
-        <x:v>Preregistration and definition freeze</x:v>
-      </x:c>
-      <x:c r="C9" s="62" t="str">
-        <x:v>Primary outcome, severe-deterioration threshold rule, universe, metrics, and final-test access rules must be frozen.</x:v>
-      </x:c>
-      <x:c r="D9" s="63" t="str">
-        <x:v>Claude Code remains blocked until this branch is approved.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="26" t="str">
-        <x:v>Literature family</x:v>
-      </x:c>
-      <x:c r="B12" s="28" t="str">
-        <x:v>Sources</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="29" t="str">
-        <x:v>Traditional disclosure baselines</x:v>
-      </x:c>
-      <x:c r="B13" s="31" t="n">
-        <x:v>17</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="29" t="str">
-        <x:v>Predictive financial text</x:v>
-      </x:c>
-      <x:c r="B14" s="31" t="n">
-        <x:v>11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="29" t="str">
-        <x:v>GenAI / AI-era disclosure</x:v>
-      </x:c>
-      <x:c r="B15" s="31" t="n">
-        <x:v>10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="29" t="str">
-        <x:v>Evidence grounding</x:v>
-      </x:c>
-      <x:c r="B16" s="31" t="n">
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="29" t="str">
-        <x:v>Drift and calibration</x:v>
-      </x:c>
-      <x:c r="B17" s="31" t="n">
-        <x:v>6</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="29" t="str">
-        <x:v>Reviews / disclosure design</x:v>
-      </x:c>
-      <x:c r="B18" s="31" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="29" t="str">
-        <x:v>AI-detector validity</x:v>
-      </x:c>
-      <x:c r="B19" s="31" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="32" t="str">
-        <x:v>Data and corpus engineering</x:v>
-      </x:c>
-      <x:c r="B20" s="34" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:D1"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82c9ebd2947f4e8d"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="32" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="105" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="35" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="55" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="26" t="str">
-        <x:v>Field / label</x:v>
+        <x:v>Metric</x:v>
       </x:c>
       <x:c r="B1" s="28" t="str">
-        <x:v>Meaning</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="54" customHeight="1">
-      <x:c r="A2" s="43" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="B2" s="45" t="str">
-        <x:v>Directly overlaps a central component and must be distinguished explicitly.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="54" customHeight="1">
-      <x:c r="A3" s="43" t="str">
-        <x:v>Medium-High</x:v>
-      </x:c>
-      <x:c r="B3" s="45" t="str">
-        <x:v>Substantial overlap with an outcome, method, or setting.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="54" customHeight="1">
-      <x:c r="A4" s="43" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="B4" s="45" t="str">
-        <x:v>Important adjacent work that changes controls, feature design, or interpretation.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="54" customHeight="1">
-      <x:c r="A5" s="43" t="str">
-        <x:v>Low / Low-Medium</x:v>
-      </x:c>
-      <x:c r="B5" s="45" t="str">
-        <x:v>Foundational literature or engineering precedent.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="54" customHeight="1">
-      <x:c r="A6" s="43" t="str">
-        <x:v>Primary verification</x:v>
-      </x:c>
-      <x:c r="B6" s="45" t="str">
-        <x:v>The journal, conference, arXiv, SSRN, or author-institution page was checked.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="54" customHeight="1">
-      <x:c r="A7" s="46" t="str">
-        <x:v>Current novelty rule</x:v>
-      </x:c>
-      <x:c r="B7" s="48" t="str">
-        <x:v>Do not claim novelty for temporal 10-K prediction, future-outcome prediction, AI-use detection, semantic drift, or controlled rewrites individually.</x:v>
+        <x:v>Value</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="29" t="str">
+        <x:v>Version</x:v>
+      </x:c>
+      <x:c r="B2" s="31" t="str">
+        <x:v>v0.3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="29" t="str">
+        <x:v>Sources</x:v>
+      </x:c>
+      <x:c r="B3" s="31" t="n">
+        <x:v>62</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="29" t="str">
+        <x:v>Added in this refresh</x:v>
+      </x:c>
+      <x:c r="B4" s="31" t="str">
+        <x:v>Choi (2026)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="29" t="str">
+        <x:v>Direct competitor audit</x:v>
+      </x:c>
+      <x:c r="B5" s="31" t="str">
+        <x:v>11 studies</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="32" t="str">
+        <x:v>Milestone 0</x:v>
+      </x:c>
+      <x:c r="B6" s="34" t="str">
+        <x:v>Complete for engineering progression</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>